<commit_message>
Condition: refresh requirement Excel
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Condition/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1617" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{673B512C-5BF3-409C-83DA-27793659718D}"/>
+  <xr:revisionPtr revIDLastSave="1810" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FA77EFC-A93B-4D05-99C9-4A0BE8DE9C03}"/>
   <bookViews>
-    <workbookView xWindow="-4044" yWindow="-17388" windowWidth="30936" windowHeight="16776" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -53,7 +53,6 @@
     <author>tc={DC3A08E9-01DD-48D1-B7F5-357810DE5428}</author>
     <author>tc={035A58F6-6A6B-4788-883F-2110C3BA07ED}</author>
     <author>tc={00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}</author>
-    <author>Shenaida Hoogland</author>
     <author>tc={065B39A6-9843-49BF-88E8-0C2BF95F8D00}</author>
   </authors>
   <commentList>
@@ -65,7 +64,7 @@
     AllergyInt heeft een andere naam conventie voor ‘Nummer’. Controleren welke juist is.</t>
       </text>
     </comment>
-    <comment ref="J19" authorId="1" shapeId="0" xr:uid="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
+    <comment ref="J21" authorId="1" shapeId="0" xr:uid="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -77,7 +76,7 @@
  evolution status - initial, interim/working, final; temporal status - current, past; episodicity status - first, new, ongoing; admission status - admission, discharge; or priority status - primary, secondary.</t>
       </text>
     </comment>
-    <comment ref="K19" authorId="2" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
+    <comment ref="K21" authorId="2" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +86,7 @@
 Kortere waardelijst</t>
       </text>
     </comment>
-    <comment ref="K23" authorId="3" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
+    <comment ref="K26" authorId="3" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +94,7 @@
     Wel in metadata!</t>
       </text>
     </comment>
-    <comment ref="E26" authorId="4" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
+    <comment ref="E29" authorId="4" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,7 +102,7 @@
     Onduidelijk welke waardelijst gehandeerd moet worden</t>
       </text>
     </comment>
-    <comment ref="B28" authorId="5" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
+    <comment ref="B31" authorId="5" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -111,7 +110,7 @@
     ter discussie</t>
       </text>
     </comment>
-    <comment ref="C28" authorId="6" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
+    <comment ref="C31" authorId="6" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -119,37 +118,7 @@
     ter discussie</t>
       </text>
     </comment>
-    <comment ref="B32" authorId="7" shapeId="0" xr:uid="{DF16D6DB-6BF2-4105-935F-CAE9E0779508}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Shenaida Hoogland:
-ter discussie</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C32" authorId="7" shapeId="0" xr:uid="{5C2BCC1D-F15F-46C8-B26A-850B59225D39}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Shenaida Hoogland:
-ter discussie</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C36" authorId="8" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
+    <comment ref="C39" authorId="7" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -162,7 +131,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="385">
   <si>
     <t>Veld</t>
   </si>
@@ -360,9 +329,6 @@
     <t>Ja</t>
   </si>
   <si>
-    <t>Condition model - EHDS Logical Information Models v1.0.0</t>
-  </si>
-  <si>
     <t>FHIR R4 resource Condition</t>
   </si>
   <si>
@@ -507,9 +473,6 @@
     <t>Subject</t>
   </si>
   <si>
-    <t>De patiënt waarover de conditie gaat</t>
-  </si>
-  <si>
     <t>Verwijzing naar Patient</t>
   </si>
   <si>
@@ -525,9 +488,6 @@
     <t>Subject of care</t>
   </si>
   <si>
-    <t xml:space="preserve">De persoon waarnaar in deze evaluatie wordt verwezen, is doorgaans de persoon op wie het medisch dossier betrekking heeft, oftewel de patiënt. </t>
-  </si>
-  <si>
     <t>Vewijzing naar Subject of Care</t>
   </si>
   <si>
@@ -537,18 +497,9 @@
     <t>CON-1.3</t>
   </si>
   <si>
-    <t>Wie heeft de conditie?</t>
-  </si>
-  <si>
-    <t>Verwijziging naar Patient of Group</t>
-  </si>
-  <si>
     <t>CON-2</t>
   </si>
   <si>
-    <t>Identificatie van object Conditie</t>
-  </si>
-  <si>
     <t>Ja (identifier)</t>
   </si>
   <si>
@@ -585,18 +536,9 @@
     <t>CON-3</t>
   </si>
   <si>
-    <t>Author</t>
-  </si>
-  <si>
-    <t>Degene die de informatie over de conditie heeft geschreven</t>
-  </si>
-  <si>
     <t>0..* Choice of types</t>
   </si>
   <si>
-    <t>Ja (recorder, 0..1)</t>
-  </si>
-  <si>
     <t>Ja (RM:other_participations)</t>
   </si>
   <si>
@@ -609,9 +551,6 @@
     <t>authorEHDSHealthProfessional</t>
   </si>
   <si>
-    <t>De zorgverlener die de informatie over de conditie heeft geschreven</t>
-  </si>
-  <si>
     <t>Verwijziging naar EHDSHealthProfessional</t>
   </si>
   <si>
@@ -630,9 +569,6 @@
     <t>authorEHDSOrganisation</t>
   </si>
   <si>
-    <t>De organisatie waaruit de informatie over de conditie afkomstig is</t>
-  </si>
-  <si>
     <t>Verwijziging naar EHDSOrganization</t>
   </si>
   <si>
@@ -648,27 +584,18 @@
     <t>authorEHDSDevice</t>
   </si>
   <si>
-    <t>Het invoerapparaat van de informatie over de conditie</t>
-  </si>
-  <si>
     <t>Verwijziging naar EHDSDevice</t>
   </si>
   <si>
     <t>CON-4</t>
   </si>
   <si>
-    <t>Datum en evt. tijd van rergistreren</t>
-  </si>
-  <si>
     <t>CON-4.1</t>
   </si>
   <si>
     <t>header.date</t>
   </si>
   <si>
-    <t>De datum en evt. tijd waarop het object is geschreven</t>
-  </si>
-  <si>
     <t>DatumTijd</t>
   </si>
   <si>
@@ -684,32 +611,6 @@
     <t>CON-4.2</t>
   </si>
   <si>
-    <t>registratiedatum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Startdatum </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Dit komt overeen met de tijd dat de concern in het patiëntendossier terecht is gekomen. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-&gt; waarom is deze datum nodig als een verplichting? Wat wil je met de informatie. moet het een timestamp tot microseconde is geregistreerd. Als we het niet kunnen vinden dan schrijven we dat ook in de variabiliteit dat mogelijk een vagere datumTijd ook mag</t>
-    </r>
-  </si>
-  <si>
     <t>Time Stamp</t>
   </si>
   <si>
@@ -723,12 +624,6 @@
   </si>
   <si>
     <t>status</t>
-  </si>
-  <si>
-    <t>De status van de conditie</t>
-  </si>
-  <si>
-    <t>Waardelijst (preferred): HL7 Condition Clinical Status Codes (active, recurrence, relapse, inactive, remission, resolved, unknown)</t>
   </si>
   <si>
     <t>Ja (clinicalStatus)</t>
@@ -749,9 +644,6 @@
 Problemen met status 'Niet actueel' verwijzen naar problemen waar de patiënt geen last meer van heeft of waar geen aanwijzingen meer voor zijn.</t>
   </si>
   <si>
-    <t>Waardelijst (actief, inactief)</t>
-  </si>
-  <si>
     <t>Spoedsamenvatting 2.2.0; Zib 2017; zib 2020</t>
   </si>
   <si>
@@ -761,25 +653,16 @@
     <t>CON-6</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
     <t>De bron van de informatie over de conditie, bijvoorbeeld de patiënt zelf</t>
   </si>
   <si>
     <t xml:space="preserve">Gecodeerde concept </t>
   </si>
   <si>
-    <t>Ja (asserter)</t>
-  </si>
-  <si>
     <t>Ja (Reference model: Information Provider) 0..1 Dit kan de patiënt zijn; een vertegenwoordiger van de patiënt, bijvoorbeeld een ouder of voogd; de behandelaar of een apparaat/software.</t>
   </si>
   <si>
     <t>CON-7</t>
-  </si>
-  <si>
-    <t>language</t>
   </si>
   <si>
     <t>De taal waarin het object is geschreven</t>
@@ -918,12 +801,6 @@
   </si>
   <si>
     <t>CON-9.3</t>
-  </si>
-  <si>
-    <t>zorgpepisode.startdatum</t>
-  </si>
-  <si>
-    <t>Bij een episode kan zowel de startdatum van de episode zelf (het begin van de contacten tussen arts en patiënt over een gezondheidskwestie) worden vastgelegd, als de begindatum van de in de episodetitel beschreven aandoening.</t>
   </si>
   <si>
     <t>CON-10</t>
@@ -1333,14 +1210,304 @@
     <t>Waarom zetten we groep er wel of niet bij? Nu niet meegenomen, maar wellicht voor in de toekomst?</t>
   </si>
   <si>
-    <t>clici</t>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.30/2026-07-29T00:00:00</t>
+  </si>
+  <si>
+    <t>Identificatie van object gezondheidstoestand</t>
+  </si>
+  <si>
+    <t>De patiënt waarover de gezondheidstoestand gaat</t>
+  </si>
+  <si>
+    <t>Verwijziging naar Patient of Groep</t>
+  </si>
+  <si>
+    <t>De persoon waarnaar in deze evaluatie wordt verwezen, is doorgaans de persoon op wie het medisch dossier betrekking heeft, oftewel de patiënt. In bepaalde omstandigheden kan het echter ook om anderen gaan, bijvoorbeeld een orgaandonor, een foetus of een familielid.</t>
+  </si>
+  <si>
+    <t>Geeft aan aan welke patiënt of groep het dossier in kader van gezondheidstoestand is gekoppeld.</t>
+  </si>
+  <si>
+    <t>CON-1.4</t>
+  </si>
+  <si>
+    <t>Nee, Kenmerken die relevant zijn voor een eenduidige definitie van het concept vormen de dataelementen van de zib. Een zib moet alle mogelijke eigenschappen van dat concept vatten voor zover relevant in gebruik van informatiesystemen binnen het zorg- en gezondheidsdomein
+Kenmerken die wel relevant zijn voor een compleet begrip, maar ook los van het concept herbruikbaar zijn worden als aparte zib middels een relaties vormgegeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nee </t>
+  </si>
+  <si>
+    <t>CON-3.4</t>
+  </si>
+  <si>
+    <t>contactpersoon als auteur</t>
+  </si>
+  <si>
+    <t>auteur</t>
+  </si>
+  <si>
+    <t>nee</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EHDSCondition.header.author</t>
+  </si>
+  <si>
+    <t>LIMS omschrijving is "	
+The author of the condition information."  Het is gemapt met FHIR: Condition.recorder: de omschrijving is "Individual who recorded the record and takes responsibility for its content." -&gt; de registratie-persoon is niet altijd ook de verantwoordelijke.  Is dit een foute mapping?</t>
+  </si>
+  <si>
+    <t>Verwijzing naar patient, zorgverlener, contactpersoon</t>
+  </si>
+  <si>
+    <t>CON-6.1</t>
+  </si>
+  <si>
+    <t>Degene die de informatie heeft verschaft en instaat voor de juistheid ervan. Dit is niet altijd zorgverlener die de gegevens invoert in het informatiesysteem, maar het kan ook de patiënt zijn of een andere betrokkene zoals bv een ouder, mantelzorger of voogd.</t>
+  </si>
+  <si>
+    <t>Informatiebron</t>
+  </si>
+  <si>
+    <t>Het apparaat waar de informatie over de conditie vandaan komt</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ja (asserter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>ja, informatiebron als basiselement</t>
+  </si>
+  <si>
+    <t>nee, niet voor elke zib klinisch relevant, en bovendien niet voor elke zib duidelijk wat hiermee bedoeld wordt, met name in relatie tot het element Auteur.</t>
+  </si>
+  <si>
+    <t>JA, auteur als basiselement</t>
+  </si>
+  <si>
+    <t>Auteur: niet voor elke zib klinisch relevant, en bovendien niet voor elke zib duidelijk wat hiermee bedoeld wordt, met name in relatie tot bron van de informatie en de vastlegger in het dossier.</t>
+  </si>
+  <si>
+    <t>Zib 2017 https://www.zibs.nl/images/2/2a/Architectuurdocument_Registratie_aan_de_bron_-_Volume_1_v1.1.pdf</t>
+  </si>
+  <si>
+    <t>Zib 2017 (https://www.zibs.nl/images/2/2a/Architectuurdocument_Registratie_aan_de_bron_-_Volume_1_v1.1.pdf)</t>
+  </si>
+  <si>
+    <t>EHDS LIM EHDSCondition 1.0.0, Zib 2017 (https://www.zibs.nl/images/2/2a/Architectuurdocument_Registratie_aan_de_bron_-_Volume_1_v1.1.pdf) 
+Spoedsamenvatting 2.2.0</t>
+  </si>
+  <si>
+    <t>EHDS LIM EHDSCondition 1.0.0
+spoedsamenvatting 2.2.0</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Ja (recorder </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 0..1)</t>
+    </r>
+  </si>
+  <si>
+    <t>ZIB 2017  (https://www.zibs.nl/images/2/2a/Architectuurdocument_Registratie_aan_de_bron_-_Volume_1_v1.1.pdf) 
+Spoedsamenvatting 2.2.0</t>
+  </si>
+  <si>
+    <t>NL-behoefte vanuit 2017:Degene op wie de informatie betrekking heeft. Vaak zal dit de patiënt zijn, maar vooral bij kleine kinderen kan het informatie over de ouder of verzorger zijn. Vooral bij de verpleegkundige overdrachten speelt b.v. bekwaamheid en betrokkenheid van mantelzorgers een rol.
+NL-behoefte komt te vervallen in zib- 2020:  impliciet is dit altijd de patiënt. In de sporadische gevallen dat de patiënt niet het onderwerp is, is dit in de betreffende zibs al expliciet gemodelleerd, zoals bijvoorbeeld in FamilieAnamnese.</t>
+  </si>
+  <si>
+    <t>Om het object uniek te identificeren in systemen</t>
+  </si>
+  <si>
+    <t>De auteur van de informatie over de gezondheidstoestand.
+NL-behoefte voor auteur, informatiebron en vastlegger komt uit 'registratie aan de bron' voor zib2017.
+NL-behoefte komt te vervallen in zib2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De organisatie waaruit de informatie over de conditie afkomstig is.
+NL-behoefte: waarom/meerwaarde vanuit de spoedsamenvatting: om verschil te maken tussen wie registreert en wie is verantwoordelijke dossierhouder; als in er kunnen verschillende zorgverleners werken bij dezelfde organisatie.-&gt; niet bekend of dit een informatiebehoefte is uit het zorgveld of uit  HL7standaard V3 CDA (custiodian en author) 
+Bij het sturen van verwijzingen, rapportages, logistieke berichten en ambulanceberichten ligt het initiatief voor gegevensuitwisseling bij de brondossierhouder (bron: https://www.nhg.org/wp-content/uploads/2023/02/Richtlijn-Gegevensuitwisseling-acute-zorg-versie-4-2022.pdf ). </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+De zorgverlener die de informatie over de conditie invoert/registreert
+NL-behoefte: Waarom/meerwaarde vanuit de spoedsamenvatting; om verschil te maken tussen wie registreert en wie is verantwoordelijke dossierhouder; Er kunnen verschillende zorgverleners werken bij dezelfde organisatie -&gt; niet bekend of dit een informatiebehoefte is uit het zorgveld of uit HL7standaard V3 CDA (custiodian en author) 
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">NL-behoefte zib2017: Degene die de informatie heeft vastgelegd. Afhankelijk van het informatiesysteem waarin de gegevens vastgelegd zijn kan dit zijn de patiënt, een </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">contactpersoon </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>of de zorgverlener.  Het is  een basiselementen. Deze zijn in de informatiemodellen van de afzonderlijke bouwstenen in de meeste gevallen niet opgenomen, maar worden wel verondersteld aanwezig te zijn. Het betreft concepten die meer technisch van aard zijn, vaak geen of weinig klinische relevantie hebben, maar voor de eenduidigheid en herleidbaarheid van de gegevens noodzakelijk zijn.
+NL-behoefte komt te vervallen in zib2020</t>
+    </r>
+  </si>
+  <si>
+    <t>Datum en evt. tijd van registreren</t>
+  </si>
+  <si>
+    <t>Datum en eventueel tijdstip van opstellen/uitgeven</t>
+  </si>
+  <si>
+    <t>Bij een episode kan zowel de startdatum van de episode zelf (het begin van de contacten tussen arts en patiënt over een gezondheidskwestie) worden vastgelegd, als de begindatum van de in de episodetitel beschreven aandoening.
+Bij template kezo-Problemobservation  is De effectiveTime, ook biologisch relevante tijd genoemd, is het tijdstip waarop de waarneming geldt voor de patient. Voor een zorgverlener die een patiënt in de kliniek vandaag ziet en waar een voorgeschiedenis van een hartaanval wordt geconstatterd die vijf jaar geleden heeft plaatsgevonden, is de effectiveTime dus vijf jaar geleden.
+de reden voor IVL_TS is onbekend</t>
+  </si>
+  <si>
+    <t>Spoedsamenvatting 2.2.0 (https://decor.nictiz.nl/pub/acutezorg/acutezorg-html-20190117T230242/tmp-2.16.840.1.113883.2.4.3.11.60.66.10.213-2015-07-03T000000.html)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zorgepisode.startdatum </t>
+  </si>
+  <si>
+    <t>probleem.startdatum</t>
+  </si>
+  <si>
+    <t>IVL_TS</t>
+  </si>
+  <si>
+    <t>Spoedsamenvatting 2.2.0 (bron: KEZO Overdracht Concern, 2.16.840.1.113883.2.4.3.11.60.66.10.212)</t>
+  </si>
+  <si>
+    <t>NL-behoefte: Dit komt overeen met de tijd dat de concern in het patiëntendossier terecht is gekomen. HIS-referentiemodel geeft aan : startdatum episode: DatumTijd=systeemdatum. Datum van het eerste contact van de patiënt met de medisch medewerker over de gezondheidskwestie van de episode. De startdatum betreft de registratie van het eerste item in de episode; cardinaliteit 1</t>
+  </si>
+  <si>
+    <t>https://referentiemodel.nhg.org/
+https://www.nhg.org/wp-content/uploads/2023/02/Richtlijn-Gegevensuitwisseling-acute-zorg-versie-4-2022.pdf</t>
+  </si>
+  <si>
+    <t>Auteur</t>
+  </si>
+  <si>
+    <t>Bron</t>
+  </si>
+  <si>
+    <t>Taal</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Condition model - EHDS Logical Information Models v1.0.0
+https://health.ec.europa.eu/publications/ehn-guideline-patient-summary_en</t>
+  </si>
+  <si>
+    <t>De status van de conditie. Requirement: eHN Guideline HDR (v1.1): A.2.6.1.7; PS (v3.4) A.2.2.2.1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">Waardelijst (preferred): HL7 Condition Clinical Status Codes (active, recurrence, relapse, inactive, remission, resolved, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>unknown?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>PAT-301</t>
+    </r>
+  </si>
+  <si>
+    <t>datumTijd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1461,6 +1628,29 @@
       <name val="Verdana"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1563,7 +1753,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1634,9 +1824,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1664,6 +1851,25 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2580,55 +2786,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2880360</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Afbeelding 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{003B378A-E260-9EB9-1F30-F75DD4C8CACD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="609600" y="5943600"/>
-          <a:ext cx="6667500" cy="3781425"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Chevy Susanto" id="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" userId="S::chevy.susanto@nictiz.nl::4e93d0cc-e599-42c6-82b7-6ffb715c7e27" providerId="AD"/>
@@ -2667,8 +2824,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N50" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A2:N50" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N53" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="A2:N53" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="4"/>
@@ -2701,8 +2858,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{87319CEB-0666-49DA-BC74-CF83CFEF5B56}" name="Tabel36" displayName="Tabel36" ref="B3:E8" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="B3:E8" xr:uid="{87319CEB-0666-49DA-BC74-CF83CFEF5B56}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{87319CEB-0666-49DA-BC74-CF83CFEF5B56}" name="Tabel36" displayName="Tabel36" ref="B3:E9" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="B3:E9" xr:uid="{87319CEB-0666-49DA-BC74-CF83CFEF5B56}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{560ECDF4-85E6-4E09-A58E-EF7D363E1023}" name="Data element" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{7F322FC5-2406-403F-A6D2-4B8A1403332A}" name="Informatiestandaard" dataDxfId="19"/>
@@ -3033,31 +3190,31 @@
   <threadedComment ref="A3" dT="2026-07-23T07:54:32.60" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{FC56F738-FB65-495B-9B48-E0F47216F010}">
     <text>AllergyInt heeft een andere naam conventie voor ‘Nummer’. Controleren welke juist is.</text>
   </threadedComment>
-  <threadedComment ref="J19" dT="2026-07-16T05:50:21.33" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
+  <threadedComment ref="J21" dT="2026-07-16T05:50:21.33" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
     <text> active
  inactive
  resolved
  in remission
  evolution status - initial, interim/working, final; temporal status - current, past; episodicity status - first, new, ongoing; admission status - admission, discharge; or priority status - primary, secondary.</text>
   </threadedComment>
-  <threadedComment ref="K19" dT="2026-07-20T09:26:12.56" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
+  <threadedComment ref="K21" dT="2026-07-20T09:26:12.56" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
     <text>1. Actief
 2. Inactief
 Kortere waardelijst</text>
   </threadedComment>
-  <threadedComment ref="K23" dT="2026-07-20T09:50:58.06" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
+  <threadedComment ref="K26" dT="2026-07-20T09:50:58.06" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
     <text>Wel in metadata!</text>
   </threadedComment>
-  <threadedComment ref="E26" dT="2026-07-20T11:55:56.61" personId="{86017760-9D2E-4C04-A548-4B0AED173840}" id="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
+  <threadedComment ref="E29" dT="2026-07-20T11:55:56.61" personId="{86017760-9D2E-4C04-A548-4B0AED173840}" id="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
     <text>Onduidelijk welke waardelijst gehandeerd moet worden</text>
   </threadedComment>
-  <threadedComment ref="B28" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
+  <threadedComment ref="B31" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
     <text>ter discussie</text>
   </threadedComment>
-  <threadedComment ref="C28" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
+  <threadedComment ref="C31" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
     <text>ter discussie</text>
   </threadedComment>
-  <threadedComment ref="C36" dT="2026-07-22T10:57:31.61" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
+  <threadedComment ref="C39" dT="2026-07-22T10:57:31.61" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
     <text>ter discussie</text>
   </threadedComment>
 </ThreadedComments>
@@ -3214,7 +3371,7 @@
       <c r="E6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="37" t="s">
+      <c r="G6" s="36" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3290,6 +3447,9 @@
       <c r="B11" s="7" t="s">
         <v>48</v>
       </c>
+      <c r="C11" s="3" t="s">
+        <v>330</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="216" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -3297,7 +3457,7 @@
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="3" t="s">
-        <v>351</v>
+        <v>326</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -3347,7 +3507,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>56</v>
       </c>
@@ -3360,8 +3520,8 @@
       <c r="D2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>60</v>
+      <c r="E2" s="4" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -3369,10 +3529,10 @@
         <v>56</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>59</v>
@@ -3386,96 +3546,100 @@
         <v>56</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>64</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>68</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E8" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
+      <c r="D9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -3534,7 +3698,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" xr:uid="{6EB8E4BD-B940-48E6-A6CE-4F11C1A8510E}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{F95A6B3D-7F5D-4E74-8C6D-B30290D6ED58}"/>
+    <hyperlink ref="E2" r:id="rId2" display="Condition model - EHDS Logical Information Models v1.0.0" xr:uid="{F95A6B3D-7F5D-4E74-8C6D-B30290D6ED58}"/>
     <hyperlink ref="E7" r:id="rId3" xr:uid="{612DD86C-3891-43E3-B27A-AA6071C8917D}"/>
     <hyperlink ref="E6" r:id="rId4" xr:uid="{104C1F39-D7B8-4AE4-9031-EE6CE3C7F3A7}"/>
     <hyperlink ref="E5" r:id="rId5" xr:uid="{B27B79EC-18DD-4070-9630-609E711CCC3B}"/>
@@ -3550,12 +3714,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
     <col min="2" max="2" width="29.33203125" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
     <col min="4" max="4" width="87.44140625" style="3" customWidth="1"/>
     <col min="5" max="5" width="26.109375" style="3" customWidth="1"/>
     <col min="6" max="6" width="18.6640625" customWidth="1"/>
@@ -3571,78 +3735,78 @@
     <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" t="s">
         <v>81</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>82</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="J2" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="K2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="71.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>95</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>96</v>
       </c>
       <c r="C3" s="19"/>
       <c r="D3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="H3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:15" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>102</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>103</v>
       </c>
       <c r="C4" s="20"/>
       <c r="D4" s="21"/>
@@ -3651,38 +3815,42 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
       <c r="I4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="K4" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+        <v>337</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>337</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="N4" s="21"/>
       <c r="O4" s="9"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="D5" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -3691,26 +3859,26 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>115</v>
+        <v>334</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -3721,24 +3889,24 @@
     </row>
     <row r="7" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>119</v>
+        <v>335</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>120</v>
+        <v>333</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -3747,287 +3915,298 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="F8" s="3"/>
+    <row r="8" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="39" t="s">
+        <v>336</v>
+      </c>
+      <c r="B8" s="40"/>
+      <c r="C8" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>124</v>
-      </c>
+      <c r="H8" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>126</v>
-      </c>
+    <row r="9" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>331</v>
+      </c>
+      <c r="C9" s="8"/>
       <c r="D9" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>128</v>
-      </c>
+        <v>362</v>
+      </c>
+      <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>106</v>
-      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3" t="s">
-        <v>130</v>
+        <v>119</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>120</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+        <v>110</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>338</v>
+      </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="C11" s="10"/>
+        <v>123</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3" t="s">
+        <v>124</v>
+      </c>
       <c r="D11" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L11" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3" t="s">
+        <v>338</v>
+      </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>142</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>377</v>
+      </c>
+      <c r="C12" s="10"/>
       <c r="D12" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="F12" s="3"/>
+        <v>363</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>146</v>
+        <v>359</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>130</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L12" s="3"/>
+        <v>354</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>353</v>
+      </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>150</v>
+        <v>365</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3" t="s">
-        <v>112</v>
+        <v>357</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L13" s="3"/>
+        <v>105</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>338</v>
+      </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>156</v>
+        <v>364</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>112</v>
+        <v>358</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L14" s="3"/>
+        <v>105</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>338</v>
+      </c>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>158</v>
+      <c r="A15" s="21" t="s">
+        <v>142</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C15" s="3"/>
+        <v>143</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
+      <c r="H15" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>162</v>
+    <row r="16" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="39" t="s">
+        <v>339</v>
+      </c>
+      <c r="B16" s="41" t="s">
+        <v>340</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>366</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>164</v>
-      </c>
+        <v>345</v>
+      </c>
+      <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3" t="s">
-        <v>112</v>
+        <v>356</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="J16" s="35" t="s">
-        <v>166</v>
+        <v>342</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>342</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
-        <v>167</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>111</v>
-      </c>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>367</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="3" t="s">
-        <v>133</v>
-      </c>
+      <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
@@ -4035,80 +4214,82 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C18" s="3"/>
+    <row r="18" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="41" t="s">
+        <v>148</v>
+      </c>
       <c r="D18" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="F18" s="3"/>
+        <v>368</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>150</v>
+      </c>
       <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
+      <c r="H18" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="J18" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>175</v>
+        <v>153</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3" t="s">
+        <v>371</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>176</v>
+        <v>375</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>177</v>
+        <v>373</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>180</v>
-      </c>
+        <v>374</v>
+      </c>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="21" t="s">
-        <v>181</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>175</v>
-      </c>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="3"/>
       <c r="D20" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>111</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="F20" s="3"/>
       <c r="G20" s="3"/>
-      <c r="H20" s="3" t="s">
-        <v>184</v>
-      </c>
+      <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
@@ -4116,406 +4297,407 @@
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="F21" s="3"/>
+    <row r="21" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A21" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E21" s="45" t="s">
+        <v>383</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
+      <c r="H21" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="10"/>
+        <v>165</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>158</v>
+      </c>
       <c r="D22" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>189</v>
+        <v>163</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>384</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="J22" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>106</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>193</v>
+        <v>378</v>
       </c>
       <c r="C23" s="10"/>
-      <c r="D23" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>164</v>
-      </c>
+      <c r="F23" s="3"/>
       <c r="G23" s="3"/>
-      <c r="H23" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="44"/>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="21" t="s">
-        <v>198</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="C24" s="24"/>
-      <c r="F24" s="3"/>
+    <row r="24" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="39"/>
+      <c r="B24" s="41"/>
+      <c r="C24" s="25" t="s">
+        <v>380</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>150</v>
+      </c>
       <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
+      <c r="H24" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="I24" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>201</v>
+        <v>350</v>
+      </c>
+      <c r="J24" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="L24" s="3"/>
+        <v>352</v>
+      </c>
+      <c r="L24" s="44" t="s">
+        <v>351</v>
+      </c>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
     </row>
-    <row r="25" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3" t="s">
-        <v>204</v>
+    <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="39" t="s">
+        <v>346</v>
+      </c>
+      <c r="B25" s="41"/>
+      <c r="C25" s="44" t="s">
+        <v>348</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>111</v>
-      </c>
+        <v>347</v>
+      </c>
+      <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3" t="s">
-        <v>112</v>
+        <v>355</v>
       </c>
       <c r="I25" s="3"/>
+      <c r="J25" s="25"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
-    <row r="26" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3" t="s">
-        <v>208</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>379</v>
+      </c>
+      <c r="C26" s="10"/>
       <c r="D26" s="3" t="s">
-        <v>209</v>
+        <v>171</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>210</v>
+        <v>172</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
+        <v>110</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>111</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="C27" s="24"/>
+      <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="21" t="s">
-        <v>216</v>
+        <v>180</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>219</v>
+        <v>183</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="C29" s="10"/>
+    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="D29" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="K29" s="3" t="s">
-        <v>226</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
-        <v>227</v>
+        <v>188</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3" t="s">
-        <v>228</v>
+        <v>189</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>229</v>
+        <v>190</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3" t="s">
-        <v>112</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="21" t="s">
-        <v>230</v>
+        <v>193</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3" t="s">
-        <v>231</v>
+        <v>194</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>232</v>
+        <v>195</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3" t="s">
-        <v>233</v>
+        <v>127</v>
       </c>
       <c r="I31" s="3"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
     </row>
-    <row r="32" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3" t="s">
-        <v>235</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C32" s="10"/>
       <c r="D32" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
+        <v>199</v>
+      </c>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>203</v>
+      </c>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="C33" s="10"/>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3" t="s">
+        <v>205</v>
+      </c>
       <c r="D33" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
+        <v>206</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="21" t="s">
-        <v>243</v>
+        <v>207</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3" t="s">
-        <v>244</v>
+        <v>208</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>245</v>
+        <v>209</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="K34" s="3" t="s">
-        <v>246</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="I34" s="3"/>
+      <c r="J34" s="33"/>
+      <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="21" t="s">
-        <v>247</v>
+    <row r="35" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>211</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3" t="s">
-        <v>248</v>
+        <v>372</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>249</v>
+        <v>369</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>171</v>
+        <v>373</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3" t="s">
-        <v>250</v>
+        <v>370</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
@@ -4524,153 +4706,138 @@
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="38" t="s">
-        <v>252</v>
-      </c>
-      <c r="D36" s="27" t="s">
-        <v>253</v>
+        <v>212</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="C36" s="10"/>
+      <c r="D36" s="3" t="s">
+        <v>214</v>
       </c>
       <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
+      <c r="G36" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>217</v>
+      </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="21" t="s">
-        <v>254</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>255</v>
-      </c>
-      <c r="C37" s="10"/>
+        <v>218</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3" t="s">
+        <v>219</v>
+      </c>
       <c r="D37" s="3" t="s">
-        <v>256</v>
+        <v>220</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>189</v>
+        <v>149</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="J37" s="22" t="s">
-        <v>258</v>
-      </c>
-      <c r="K37" s="3"/>
+        <v>110</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>221</v>
+      </c>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A38" s="21" t="s">
-        <v>259</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="C38" s="10"/>
+        <v>222</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3" t="s">
+        <v>223</v>
+      </c>
       <c r="D38" s="3" t="s">
-        <v>261</v>
+        <v>224</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>262</v>
+        <v>154</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I38" s="36" t="s">
-        <v>263</v>
-      </c>
-      <c r="J38" s="36" t="s">
-        <v>264</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>266</v>
-      </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>269</v>
-      </c>
+    <row r="39" spans="1:14" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
       <c r="H39" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>271</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="21" t="s">
-        <v>272</v>
+        <v>229</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>273</v>
+        <v>230</v>
       </c>
       <c r="C40" s="10"/>
       <c r="D40" s="3" t="s">
-        <v>274</v>
+        <v>231</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>275</v>
+        <v>168</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>277</v>
+        <v>232</v>
+      </c>
+      <c r="J40" s="22" t="s">
+        <v>233</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
@@ -4679,80 +4846,96 @@
     </row>
     <row r="41" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3" t="s">
-        <v>279</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="C41" s="10"/>
       <c r="D41" s="3" t="s">
-        <v>280</v>
+        <v>236</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>237</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
+        <v>110</v>
+      </c>
+      <c r="I41" s="35" t="s">
+        <v>238</v>
+      </c>
+      <c r="J41" s="35" t="s">
+        <v>239</v>
+      </c>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="21" t="s">
-        <v>281</v>
-      </c>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3" t="s">
-        <v>282</v>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="C42" s="10"/>
       <c r="D42" s="3" t="s">
-        <v>283</v>
+        <v>242</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>243</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G42" s="3"/>
+        <v>150</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>244</v>
+      </c>
       <c r="H42" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
+        <v>110</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>246</v>
+      </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
     </row>
-    <row r="43" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="21" t="s">
-        <v>284</v>
+        <v>247</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>285</v>
+        <v>248</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="3" t="s">
-        <v>286</v>
+        <v>249</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>287</v>
+        <v>250</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="J43" s="26" t="s">
-        <v>289</v>
+        <v>251</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>252</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
@@ -4760,18 +4943,25 @@
       <c r="N43" s="3"/>
     </row>
     <row r="44" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A44" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>291</v>
-      </c>
-      <c r="C44" s="10"/>
-      <c r="F44" s="3"/>
+      <c r="A44" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>150</v>
+      </c>
       <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
+      <c r="H44" s="3" t="s">
+        <v>210</v>
+      </c>
       <c r="I44" s="3"/>
-      <c r="J44" s="26"/>
+      <c r="J44" s="3"/>
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3"/>
@@ -4779,93 +4969,74 @@
     </row>
     <row r="45" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="21" t="s">
-        <v>292</v>
-      </c>
-      <c r="B45" s="10"/>
-      <c r="C45" s="22" t="s">
-        <v>293</v>
+        <v>256</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3" t="s">
+        <v>257</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>295</v>
+        <v>258</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="G45" s="3"/>
       <c r="H45" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="J45" s="22" t="s">
-        <v>297</v>
-      </c>
-      <c r="K45" s="27" t="s">
-        <v>298</v>
-      </c>
-      <c r="L45" s="27"/>
-      <c r="M45" s="27"/>
+        <v>210</v>
+      </c>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="B46" s="3"/>
-      <c r="C46" s="22" t="s">
-        <v>300</v>
-      </c>
+    <row r="46" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A46" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="C46" s="10"/>
       <c r="D46" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>302</v>
+        <v>261</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>262</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I46" s="3"/>
-      <c r="J46" s="3"/>
-      <c r="K46" s="27"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
+        <v>110</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="J46" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
     <row r="47" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="21" t="s">
-        <v>303</v>
+      <c r="A47" s="9" t="s">
+        <v>265</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>304</v>
+        <v>266</v>
       </c>
       <c r="C47" s="10"/>
-      <c r="D47" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>128</v>
-      </c>
+      <c r="F47" s="3"/>
       <c r="G47" s="3"/>
-      <c r="H47" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I47" s="36" t="s">
-        <v>307</v>
-      </c>
-      <c r="J47" s="22" t="s">
-        <v>308</v>
-      </c>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="26"/>
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3"/>
@@ -4873,102 +5044,196 @@
     </row>
     <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="21" t="s">
-        <v>309</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>310</v>
-      </c>
-      <c r="C48" s="10"/>
+        <v>267</v>
+      </c>
+      <c r="B48" s="10"/>
+      <c r="C48" s="22" t="s">
+        <v>268</v>
+      </c>
       <c r="D48" s="3" t="s">
-        <v>311</v>
+        <v>269</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>312</v>
+        <v>270</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>313</v>
+        <v>150</v>
       </c>
       <c r="G48" s="3"/>
       <c r="H48" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="J48" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="K48" s="3"/>
-      <c r="L48" s="3"/>
-      <c r="M48" s="3"/>
+        <v>271</v>
+      </c>
+      <c r="J48" s="22" t="s">
+        <v>272</v>
+      </c>
+      <c r="K48" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="L48" s="27"/>
+      <c r="M48" s="27"/>
       <c r="N48" s="3"/>
     </row>
-    <row r="49" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="21" t="s">
-        <v>316</v>
-      </c>
-      <c r="B49" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="C49" s="30"/>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A49" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="22" t="s">
+        <v>275</v>
+      </c>
       <c r="D49" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>262</v>
+        <v>276</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>277</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I49" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="J49" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="K49" s="3"/>
-      <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
+        <v>210</v>
+      </c>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="27"/>
+      <c r="L49" s="17"/>
+      <c r="M49" s="17"/>
       <c r="N49" s="3"/>
     </row>
-    <row r="50" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="9" t="s">
-        <v>320</v>
-      </c>
-      <c r="B50" t="s">
-        <v>321</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>322</v>
+    <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="C50" s="10"/>
+      <c r="D50" s="3" t="s">
+        <v>280</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="H50" t="s">
-        <v>324</v>
-      </c>
-      <c r="I50" t="s">
-        <v>325</v>
-      </c>
-      <c r="J50" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B54" s="31"/>
-      <c r="C54" s="31"/>
-    </row>
-    <row r="55" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B55" s="32"/>
-      <c r="C55" s="33"/>
-    </row>
-    <row r="56" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="31"/>
-      <c r="C56" s="31"/>
+        <v>281</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I50" s="35" t="s">
+        <v>282</v>
+      </c>
+      <c r="J50" s="22" t="s">
+        <v>283</v>
+      </c>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+    </row>
+    <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="21" t="s">
+        <v>284</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="C51" s="10"/>
+      <c r="D51" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+    </row>
+    <row r="52" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="B52" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C52" s="29"/>
+      <c r="D52" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+    </row>
+    <row r="53" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="B53" t="s">
+        <v>296</v>
+      </c>
+      <c r="D53" s="23" t="s">
+        <v>297</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H53" t="s">
+        <v>299</v>
+      </c>
+      <c r="I53" t="s">
+        <v>300</v>
+      </c>
+      <c r="J53" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B57" s="30"/>
+      <c r="C57" s="30"/>
+    </row>
+    <row r="58" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B58" s="31"/>
+      <c r="C58" s="32"/>
+    </row>
+    <row r="59" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="30"/>
+      <c r="C59" s="30"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -4997,48 +5262,48 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>328</v>
+        <v>303</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>330</v>
+        <v>305</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>331</v>
+        <v>306</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -5055,7 +5320,7 @@
     <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>332</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -5075,7 +5340,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>333</v>
+        <v>308</v>
       </c>
       <c r="B1" t="s">
         <v>53</v>
@@ -5083,15 +5348,15 @@
     </row>
     <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>334</v>
+        <v>309</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>335</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>336</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -5104,7 +5369,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E8E4E8-143C-4C64-99FB-1306F2338EFB}">
-  <dimension ref="A2:J8"/>
+  <dimension ref="A2:J9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.6640625" style="3" customWidth="1"/>
@@ -5115,7 +5380,7 @@
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B2" s="15" t="s">
-        <v>337</v>
+        <v>312</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -5123,52 +5388,52 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B3" s="16" t="s">
-        <v>338</v>
+        <v>313</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>339</v>
+        <v>314</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="14" t="s">
-        <v>341</v>
+        <v>316</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>342</v>
+        <v>317</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>343</v>
+        <v>318</v>
       </c>
       <c r="E4" s="14"/>
     </row>
     <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="14" t="s">
-        <v>344</v>
+        <v>319</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>345</v>
+        <v>320</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>346</v>
+        <v>321</v>
       </c>
       <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21"/>
       <c r="B6" s="3" t="s">
-        <v>304</v>
+        <v>279</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>347</v>
+        <v>322</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>348</v>
+        <v>323</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5178,33 +5443,42 @@
     </row>
     <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="14" t="s">
-        <v>349</v>
+        <v>324</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>347</v>
+        <v>322</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>350</v>
+        <v>325</v>
       </c>
       <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B8" s="14" t="s">
-        <v>353</v>
+        <v>328</v>
       </c>
       <c r="C8" s="14"/>
-      <c r="D8" s="39" t="s">
-        <v>352</v>
+      <c r="D8" s="38" t="s">
+        <v>327</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>354</v>
-      </c>
+        <v>329</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="B9" s="42"/>
+      <c r="C9" s="42" t="s">
+        <v>343</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>344</v>
+      </c>
+      <c r="E9" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Condition: concept tab aligned with other gbbs
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichalCiszewski\Documents\Github\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1320D0F2-528E-4561-A815-608E3850C934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455916BA-1B1A-461D-977E-85F4A305936A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
-    <sheet name="Concept" sheetId="2" r:id="rId2"/>
+    <sheet name="Concept" sheetId="9" r:id="rId2"/>
     <sheet name="Bronnen" sheetId="6" r:id="rId3"/>
     <sheet name="Informatiebehoefte" sheetId="1" r:id="rId4"/>
     <sheet name="Ongedekte informatiebehoefte" sheetId="3" r:id="rId5"/>
@@ -22,6 +22,12 @@
     <sheet name="Basismodel" sheetId="7" r:id="rId7"/>
     <sheet name="Ter discussie" sheetId="8" r:id="rId8"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId9"/>
+  </externalReferences>
+  <definedNames>
+    <definedName name="Informatiebron">[1]!Tabel3[Naam bron]</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -130,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="353">
   <si>
     <t>Veld</t>
   </si>
@@ -138,151 +144,52 @@
     <t>Beschrijving</t>
   </si>
   <si>
-    <t>Invulling (zelf beschreven op basis van openEHR, FHIR R4 en EHDS LIM)</t>
-  </si>
-  <si>
-    <t>Bronnen</t>
-  </si>
-  <si>
-    <t>a.d.h.v. keuze FHIR als basismodel</t>
-  </si>
-  <si>
-    <t>a.d.h.v. keuze OpenEHR als basismodel</t>
-  </si>
-  <si>
     <t>Conceptbeschrijving</t>
   </si>
   <si>
-    <t>[De definitie of beschrijving van het concept.]</t>
-  </si>
-  <si>
     <t>Een conditie beschrijft een klinisch relevante gezondheidstoestand, diagnose, probleem, aandoening of andere gezondheidsituatie die betrekking heeft op de gezondheid en/of het welzijn van de patiënt. Deze toestand kan benoemd zijn door de patiënt, gerelateerd persoon of door de zorgverlener. De gezondheidstoestand kan aanleiding geven tot behandeling, monitoring of vervolgbeleid.</t>
   </si>
   <si>
-    <t>Samengesteld uit EHDS LIM EHDSCondition v1.0.0; FHIR R4 Condition; openEHR problem/Diagnosis v1.5.0; zib Probleem 2020</t>
-  </si>
-  <si>
-    <t>Een klinische aandoening, probleem, diagnose of andere gebeurtenis, situatie, kwestie of klinisch concept dat aanleiding geeft tot zorg.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Details over een specifieke gezondheidstoestand, letsel, handicap of ander probleem dat van invloed is op het fysieke, mentale en/of sociale welzijn van een individu.
-Opmerking: In de praktijk is het niet eenvoudig om een ​​duidelijke scheiding te maken tussen de omvang van een probleem en een diagnose. Voor klinische documentatie met dit archetype worden probleem en diagnose beschouwd als een continuüm, waarbij toenemende mate van detail en ondersteunend bewijs doorgaans meer gewicht toekennen aan het label 'diagnose'.
-</t>
-  </si>
-  <si>
-    <t>EDHS LIM: Model for a clinical condition, problem, diagnosis, or other event, situation, or issue that has risen to a level of concern.
-OpenEHR: 
-ChatGPT samenvatting van FHIR R4 resource: Model voor klinisch relevante gezondheidstoestand van een patiënt die door een zorgverlener zijn beoordeeld of vastgesteld. Dit kan een diagnose, gezondheidsprobleem, zorgvraag of andere gezondheidssituatie zijn die aanleiding geeft tot behandeling, monitoring of vervolgbeleid.
-Zib Probleem 2020: Een probleem beschrijft een toestand met betrekking tot de gezondheid en/of het welzijn van een individu. Deze toestand kan zijn benoemd door de betroffene (de patiënt) zelf (een klacht), of door zijn of haar zorgverlener (onder andere een diagnose). De toestand kan aanleiding zijn voor diagnostisch of therapeutisch beleid.
-Een probleem omvat allerlei soorten medische of verpleegkundige gegevens, die een gezondheidsprobleem representeren. Een probleem kan verschillende typen gezondheidsproblemen representeren: symptoom, klacht, diagnose, functionele beperking, complicatie. 
-OpenEHR: Details over een specifieke gezondheidstoestand, letsel, handicap of ander probleem dat van invloed is op het fysieke, mentale en/of sociale welzijn van een persoon.</t>
-  </si>
-  <si>
     <t>Doel</t>
   </si>
   <si>
-    <t>[De doelen en redenen om het concept vast te leggen en/of uit te wisselen.]</t>
-  </si>
-  <si>
     <t xml:space="preserve">Een overzicht van gezondheidstoestanden/diagnoses/aandoeningen van de patient. </t>
   </si>
   <si>
-    <t>Gedestileerd uit de conceptbeschrijving</t>
-  </si>
-  <si>
-    <t>Het doel van het concept is het eenduidig vastleggen en uitwisselen van een klinisch relevante diagnose, aandoening, gezondheidstoestand of ander zorgpunt van een patiënt. Dit ondersteunt nader onderzoek, behandeling, monitoring en overdracht van zorg, ook wanneer het gaat om een niet-negatieve gezondheidstoestand, zoals zwangerschap, of om een toestand die het gevolg is van een eerdere ingreep.</t>
-  </si>
-  <si>
-    <t>Voor het vastleggen van details over een enkel, geïdentificeerd gezondheidsprobleem of diagnose.
-De beoogde reikwijdte van een gezondheidsprobleem wordt in de context van klinische documentatie bewust ruim gehouden, zodat alle reële of vermeende zorgen die het welzijn van een persoon in welke mate dan ook negatief kunnen beïnvloeden, kunnen worden vastgelegd. Een gezondheidsprobleem kan worden geïdentificeerd door de persoon zelf, een mantelzorger of een zorgverlener. Een diagnose wordt echter daarnaast gedefinieerd op basis van objectieve klinische criteria en wordt doorgaans alleen vastgesteld door een zorgverlener.</t>
-  </si>
-  <si>
     <t>Gebruiksscenario(’s)</t>
-  </si>
-  <si>
-    <t>[Geeft aan in welke context(en) het concept wordt gebruikt. Geef voorbeelden van gebruik in informatiestandaarden.]</t>
   </si>
   <si>
     <t>Een overzicht van gezondheidstoestanden/diagnoses/aandoeningen van de patient. Het wordt gebruikt in de informatiestandaarden BgZ-MSZ, Eerstelijnszorg, .. 
 Conditie kan worden gebruikt om het gezondheidsprobleem in een zorgepisode te duiden.</t>
   </si>
   <si>
-    <t>Afkomstig uit informatiestandaard BgZ-MSZ, informatiestandaard Acute Zorg</t>
-  </si>
-  <si>
-    <t>Het kan worden gebruikt om informatie vast te leggen over een ziekte of aandoening die is vastgesteld op basis van klinische redenering over pathologische en pathofysiologische bevindingen (diagnose); over gezondheidsproblemen of -situaties die een zorgverlener als schadelijk of potentieel schadelijk beschouwt en die nader onderzoek en behandeling vereisen (probleem); of over andere gezondheidsproblemen of -situaties die mogelijk voortdurende monitoring en/of behandeling behoeven (gezondheidsprobleem/-zorgpunt).
-De 'Condition'-resource kan worden gebruikt om een ​​bepaalde gezondheidstoestand van een patiënt vast te leggen die doorgaans niet als een negatieve uitkomst wordt beschouwd, zoals zwangerschap. De 'Condition'-resource kan ook worden gebruikt om een ​​aandoening of toestand vast te leggen die volgt op een ingreep, zoals de status van 'onderbeenamputatiepatiënt' na een amputatieprocedure.
-Spoedsamenvatting 2.2.0, bij het opstellen van de episodes en problemen 
-BgZ-MSZ: bij klachten en diagnoses
-eOverdracht: problemen
-Eerstelijnszorg: problemen</t>
-  </si>
-  <si>
-    <t>Dit archetype kan in veel contexten worden gebruikt. Bijvoorbeeld om een ​​probleem of een klinische diagnose vast te leggen tijdens een consult; om een ​​permanente probleemlijst aan te vullen; of om een ​​samenvattende verklaring op te nemen in een ontslagbrief.</t>
-  </si>
-  <si>
     <t>Representatie</t>
   </si>
   <si>
-    <t>[Beschrijf hier wat er voor de dossiervorming belangrijk is rondom de levenscyclus en instantiaties van het concept.]</t>
-  </si>
-  <si>
     <t>Een gezondheidsstoestand heeft een start en kan een einddatum hebben, maar hoeft niet. Het kan gevlagt zijn om in de probleemlijst van de patient aanwezig te blijven, ook al is de gezondheidsstoestand opgeheven.</t>
   </si>
   <si>
-    <t>Gedestileerd uit de data-elementen van de EHDS LIM EHDSCondition v1.0.0</t>
-  </si>
-  <si>
-    <t>Een instantiatie beschrijft één klinisch relevante conditie bij een patiënt. Veranderingen in status of zekerheid worden in dezelfde registratie bijgewerkt; voor een andere conditie of afzonderlijke episode wordt een nieuwe instantiatie gemaakt. Beëindigde of weerlegde condities blijven als historie beschikbaar.</t>
-  </si>
-  <si>
-    <t>kijken hoe openEHR erover denkt met evoluerende diagnose van de patient.</t>
-  </si>
-  <si>
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>[Alle bekende synoniemen voor het concept.]</t>
-  </si>
-  <si>
     <t>episode, diagnose, aandoening, probleem, klacht(als het geen onderdeel is van de aandoening), functionele beperking, complicatie, symptoom(als het geen onderdeel is van de aandoening)</t>
   </si>
   <si>
     <t>Juist gebruik</t>
   </si>
   <si>
-    <t>[Beschrijf hier waarvoor het concept wél bedoeld is].</t>
-  </si>
-  <si>
     <t>Voor het vastleggen van diagnoses, probleem, en andere situaties van de patiënt die geen negatieve uitkomst hebben. zoals een zwangerschap.</t>
   </si>
   <si>
-    <t>Het concept is bedoeld voor het vastleggen van een klinisch relevante aandoening, diagnose, probleem, gezondheidstoestand, risico of zorgpunt dat beoordeling, behandeling of monitoring vereist.</t>
-  </si>
-  <si>
-    <t>Te gebruiken voor het vastleggen van details over een enkel, geïdentificeerd gezondheidsprobleem of diagnose.
-Duidelijke definities die onderscheid maken tussen een 'probleem' en een 'diagnose' zijn in de praktijk vrijwel onmogelijk - we kunnen niet betrouwbaar vaststellen wanneer een probleem als een diagnose moet worden beschouwd. 
-Voor klinische documentatie met dit archetype worden probleem en diagnose beschouwd als een continuüm, waarbij toenemende mate van detail en ondersteunend bewijsmateriaal doorgaans meer gewicht in de schaal legt voor de benaming 'diagnose'. In dit archetype is het niet nodig om de aandoening te classificeren als een 'probleem' of 'diagnose'.</t>
-  </si>
-  <si>
     <t>Onjuist gebruik</t>
   </si>
   <si>
-    <t>[Beschrijf hier waar het concept niet voor bedoeld is, en geef waar mogelijk aan welk concept er wel geschikt voor is.]</t>
-  </si>
-  <si>
     <t>Het wordt niet gebruikt om de functionele status, bijvoorbeeld vermogen tot ADL, vast te leggen. Het wordt niet gebruikt voor symptomen die je observeert of uitvraagt, met andere woorden wanneer een symptoom bijdraagt aan de aandoening, dient het niet opgenomen te worden als condition.</t>
   </si>
   <si>
-    <t>Het concept is niet bedoeld voor losse metingen, bevindingen of kortdurende symptomen; gebruik hiervoor Observation. Het is ook niet bedoeld om de uitgevoerde ingreep zelf vast te leggen; gebruik daarvoor Procedure. Voor allergieën en intoleranties die klinische beslisondersteuning moeten activeren, is AllergyIntolerance het aangewezen concept. Een blijvende toestand na een ingreep kan wel als conditie worden vastgelegd.</t>
-  </si>
-  <si>
     <t>Referenties</t>
   </si>
   <si>
-    <t>[Relevante bronstandaarden of informatiebronnen die het ontwerp en de scope van het concept hebben beïnvloed.]</t>
-  </si>
-  <si>
     <t>EHDS LIM EHDSCondition v1.0.0; FHIR R4 resource Condition; openEHR Problem/Diagnosis 1.5.0</t>
   </si>
   <si>
@@ -290,15 +197,6 @@
   </si>
   <si>
     <t>ART-DECOR-id</t>
-  </si>
-  <si>
-    <t>[Het id op ART-DECOR van het afsprakenmodel, bv 2.16.840.1.113883.2.4.3.11.60.153.4.12/2026-06-04T00:00:00]</t>
-  </si>
-  <si>
-    <t>Keuze Basismodel</t>
-  </si>
-  <si>
-    <t>Concept-sheet is opgemaakt met spelregel: https://nictiz.atlassian.net/browse/DAGIM-72</t>
   </si>
   <si>
     <t>Type bron</t>
@@ -1164,40 +1062,6 @@
   </si>
   <si>
     <t>niet in FHIR wel in openEHR. komt hier een extension voor? Device wordt nu uitgewerkt in team carefuel</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Na analyse blijkt FHIR beste keus, want:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  [hier nog even de volwassenheid van FHIR-basismodel en openEHR neerzetten]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>- category geen mapping heeft op openEHR en wel een mapping op FHIR
-- diagnosisAssertionStatus waardelijst komt niet precies overeen bij openEHR, wel in FHIR
-- stage komt niet precies overeen in openEHR, namelijk via extensie / uitbreiding van archetype Specific Details (cluster?), wel in FHIR
-- nadereSpecificatieProbleemNaam heeft in ZIBFHIR-145 een mapping gekregen op FHIR, maar is duidelijker in openEHR gemodelleerd als "variant" (echter variant is specifieker, dan LIMS/ZIB wil duiden )
--specialistcontact: in openEHR is het onduidelijk, mogelijk other participants mits je aan kan geven dat het een voorkeurscontactpersoon is. in FHIR ook niet ideaal, namelijk note.text of via careteam.reason</t>
-    </r>
   </si>
   <si>
     <t>Indicates the patient or group who the condition record is associated with.</t>
@@ -1506,7 +1370,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1650,8 +1514,34 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1672,12 +1562,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1689,7 +1573,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1723,36 +1607,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1765,9 +1625,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1795,9 +1652,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1836,16 +1690,15 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1854,12 +1707,33 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="20">
     <dxf>
       <font>
         <color rgb="FF000000"/>
@@ -1951,52 +1825,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2062,6 +1890,27 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2194,7 +2043,7 @@
       <xdr:rowOff>223837</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>2181225</xdr:rowOff>
@@ -2204,7 +2053,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7E9BA32-9F57-9DBE-09F8-19BB04854D12}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECAA1215-2A99-4248-92C1-D8603DD25A54}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2213,7 +2062,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="161925" y="223837"/>
-          <a:ext cx="6705600" cy="1957388"/>
+          <a:ext cx="6802755" cy="1957388"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2770,6 +2619,40 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Uitleg"/>
+      <sheetName val="Concept"/>
+      <sheetName val="Bronnen informatiebehoefte"/>
+      <sheetName val="Niet geconsolideerde info"/>
+      <sheetName val="Informatiebehoefte"/>
+      <sheetName val="Ongedekte informatiebehoefte"/>
+      <sheetName val="Overwegingen voor de toekomst"/>
+      <sheetName val="zib-centrum JIRA"/>
+      <sheetName val="Basismodel "/>
+      <sheetName val="Template informatiebehoefte - A"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Chevy Susanto" id="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" userId="S::chevy.susanto@nictiz.nl::4e93d0cc-e599-42c6-82b7-6ffb715c7e27" providerId="AD"/>
@@ -2779,58 +2662,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7AAA9086-205B-4EC4-8920-A2DD04D02676}" name="Tabel2" displayName="Tabel2" ref="A2:F13" totalsRowShown="0">
-  <autoFilter ref="A2:F13" xr:uid="{7AAA9086-205B-4EC4-8920-A2DD04D02676}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{BDCFF82A-D4BE-440B-90DF-AA26F6831D5C}" name="Veld"/>
-    <tableColumn id="2" xr3:uid="{77503B9E-152C-4B39-87F4-D4FBBF1B3BDA}" name="Beschrijving" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{DAF348AE-F547-4357-9E3C-18B833059F60}" name="Invulling (zelf beschreven op basis van openEHR, FHIR R4 en EHDS LIM)" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{6782DEBA-8C39-4E2C-BBC2-2CD68FCA1048}" name="Bronnen" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{B530BE2A-715C-42B8-BFE1-95637D35484B}" name="a.d.h.v. keuze FHIR als basismodel"/>
-    <tableColumn id="6" xr3:uid="{1CF171A1-4997-44CE-A155-D2A5B879A058}" name="a.d.h.v. keuze OpenEHR als basismodel"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}" name="Tabel3" displayName="Tabel3" ref="A1:E17" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:E17" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{2D5F85E5-856C-4A15-8C5D-D8D344B8F13C}" name="Type bron" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{062A7D5A-6D4F-45DD-9A5C-7A2D82A1266A}" name="Naam bron" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{24E64AAE-4BAD-402C-98B7-B46BE371B39E}" name="Toelichting" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{98DE6918-807C-41E0-ACBA-1E2221CF05FC}" name="Informatiebehoefte verwerkt in sheet 'informatiebeheofte'" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{8CFF4D4C-ABDD-49BC-8B49-237193168687}" name="Link naar bron informatie" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}" name="Tabel3" displayName="Tabel3" ref="A1:E17" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:E17" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2D5F85E5-856C-4A15-8C5D-D8D344B8F13C}" name="Type bron" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{062A7D5A-6D4F-45DD-9A5C-7A2D82A1266A}" name="Naam bron" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{24E64AAE-4BAD-402C-98B7-B46BE371B39E}" name="Toelichting" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{98DE6918-807C-41E0-ACBA-1E2221CF05FC}" name="Informatiebehoefte verwerkt in sheet 'informatiebeheofte'" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{8CFF4D4C-ABDD-49BC-8B49-237193168687}" name="Link naar bron informatie" dataDxfId="6"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N53" totalsRowShown="0" headerRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N53" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="A2:N53" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="10"/>
     <tableColumn id="12" xr3:uid="{721FE94A-B8C9-44E1-A03C-56E48CDCE2A3}" name="data-element"/>
-    <tableColumn id="3" xr3:uid="{12776FCA-6A89-4E9E-907F-2E30F0D43DA3}" name="Omschrijving" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{9E28C4DB-2A8B-484B-80F1-321440976652}" name="Variabiliteit" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{12776FCA-6A89-4E9E-907F-2E30F0D43DA3}" name="Omschrijving" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{9E28C4DB-2A8B-484B-80F1-321440976652}" name="Variabiliteit" dataDxfId="8"/>
     <tableColumn id="5" xr3:uid="{6FA3E114-7382-4230-B15E-A8DB28B8CE4B}" name="Aanwezigheid"/>
     <tableColumn id="6" xr3:uid="{E8FFDBDF-8B88-4089-89D0-252402D12764}" name="Verleden/heden/toekomst"/>
     <tableColumn id="7" xr3:uid="{BB9C62AB-9839-431A-90A2-B6A6D70DF1FB}" name="Herkomst"/>
     <tableColumn id="8" xr3:uid="{6BE87E7D-EFAE-42FD-9334-11E5EBAC9DC3}" name="Komt het in FHIR R4 voor?"/>
     <tableColumn id="9" xr3:uid="{C6EE00AA-2B37-4BE3-B349-AF61C6E68575}" name="Komt het in openEHR voor?"/>
     <tableColumn id="10" xr3:uid="{943D4BF3-315C-41FB-99E4-8DB8C54604A4}" name="Komt voor in ZIBProbleem-v4.4? (2020)"/>
-    <tableColumn id="14" xr3:uid="{8B1A7EB4-D690-4A36-9698-ACA592C2A715}" name="Komt voor in ZIBProbleem? (2017)" dataDxfId="17"/>
-    <tableColumn id="13" xr3:uid="{51A57E0A-A216-45BB-973D-E0D8C72BEEEC}" name="Komt voor in ZIBProbleem? (2024)" dataDxfId="16"/>
+    <tableColumn id="14" xr3:uid="{8B1A7EB4-D690-4A36-9698-ACA592C2A715}" name="Komt voor in ZIBProbleem? (2017)" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{51A57E0A-A216-45BB-973D-E0D8C72BEEEC}" name="Komt voor in ZIBProbleem? (2024)" dataDxfId="6"/>
     <tableColumn id="11" xr3:uid="{E7EDB106-7E3F-4122-A864-3B3AE59C9D87}" name="Opmerking"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D40E6C54-E02A-43EF-B5CE-2ED10C0E81CC}" name="Tabel4" displayName="Tabel4" ref="A1:B10" totalsRowShown="0">
   <autoFilter ref="A1:B10" xr:uid="{D40E6C54-E02A-43EF-B5CE-2ED10C0E81CC}"/>
   <tableColumns count="2">
@@ -2841,7 +2709,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{87319CEB-0666-49DA-BC74-CF83CFEF5B56}" name="Tabel36" displayName="Tabel36" ref="B3:E9" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="B3:E9" xr:uid="{87319CEB-0666-49DA-BC74-CF83CFEF5B56}"/>
   <tableColumns count="4">
@@ -3240,225 +3108,170 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
-  <dimension ref="A1:G13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95E1B5B8-C013-4DD1-9595-10AFF6D9F062}">
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="62.33203125" customWidth="1"/>
-    <col min="3" max="3" width="76.44140625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="30" style="3" customWidth="1"/>
-    <col min="5" max="5" width="45.5546875" customWidth="1"/>
-    <col min="6" max="6" width="64.109375" customWidth="1"/>
-    <col min="7" max="7" width="129.5546875" customWidth="1"/>
+    <col min="2" max="2" width="29.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="B3" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="C3" s="39"/>
+      <c r="D3" s="40"/>
+    </row>
+    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="B4" s="38" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="219.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C4" s="39"/>
+      <c r="D4" s="40"/>
+    </row>
+    <row r="5" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B5" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C5" s="39"/>
+      <c r="D5" s="40"/>
+    </row>
+    <row r="6" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="B6" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="C6" s="39"/>
+      <c r="D6" s="40"/>
+    </row>
+    <row r="7" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="B7" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="D7" s="41"/>
+    </row>
+    <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="165" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B8" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C8" s="39"/>
+      <c r="D8" s="42"/>
+    </row>
+    <row r="9" spans="1:4" ht="144" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B9" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C9" s="39"/>
+      <c r="D9" s="41"/>
+    </row>
+    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="B10" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="360" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C10" s="39"/>
+      <c r="D10" s="40"/>
+    </row>
+    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="36" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="156" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="216" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="3" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" s="7"/>
+      <c r="B11" t="s">
+        <v>298</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="40"/>
+    </row>
+    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C12" s="39"/>
+      <c r="D12" s="40"/>
+    </row>
+    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B13" s="43"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="40"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B14" s="5"/>
+      <c r="C14" s="44"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B15" s="5"/>
+      <c r="C15" s="44"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16" s="43"/>
+      <c r="C16" s="44"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B17" s="43"/>
+      <c r="C17" s="44"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="43"/>
+      <c r="C18" s="39"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B19" s="43"/>
+      <c r="C19" s="44"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" s="43"/>
+      <c r="C20" s="44"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="39"/>
+      <c r="C21" s="44"/>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B22" s="43"/>
+      <c r="C22" s="44"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B23" s="43"/>
+      <c r="C23" s="44"/>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B24" s="43"/>
+      <c r="C24" s="39"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E10" r:id="rId1" display="https://www.hl7.org/fhir/R4/condition.html" xr:uid="{6169B330-2124-4ACC-9C33-24AFE1D4848F}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
-  </tableParts>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3476,154 +3289,154 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>381</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>46</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="5" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="5" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="5" t="s">
-        <v>73</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>376</v>
+        <v>344</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -3719,122 +3532,122 @@
     <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>84</v>
+        <v>51</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>89</v>
+        <v>56</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>58</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="71.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="C3" s="19"/>
+        <v>63</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="17"/>
       <c r="D3" s="1" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>97</v>
+        <v>66</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>99</v>
+        <v>68</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+      <c r="A4" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="18"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
       <c r="I4" s="3" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="K4" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="L4" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="M4" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="N4" s="21"/>
-      <c r="O4" s="9"/>
+        <v>73</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="L4" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="M4" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="N4" s="19"/>
+      <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>107</v>
+      <c r="A5" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>76</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>332</v>
+        <v>300</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -3844,25 +3657,25 @@
       <c r="N5" s="3"/>
     </row>
     <row r="6" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8" t="s">
-        <v>112</v>
+      <c r="A6" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
+        <v>81</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>334</v>
+        <v>302</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>113</v>
+        <v>82</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>114</v>
+        <v>83</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -3872,25 +3685,25 @@
       <c r="N6" s="3"/>
     </row>
     <row r="7" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8" t="s">
-        <v>107</v>
+      <c r="A7" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>76</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>335</v>
+        <v>303</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>333</v>
+        <v>301</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -3900,25 +3713,25 @@
       <c r="N7" s="3"/>
     </row>
     <row r="8" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>336</v>
-      </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8" t="s">
-        <v>308</v>
+      <c r="A8" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>277</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>361</v>
+        <v>329</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>360</v>
+        <v>328</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -3928,15 +3741,15 @@
       <c r="N8" s="3"/>
     </row>
     <row r="9" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>331</v>
-      </c>
-      <c r="C9" s="8"/>
+      <c r="A9" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>299</v>
+      </c>
+      <c r="C9" s="7"/>
       <c r="D9" s="3" t="s">
-        <v>362</v>
+        <v>330</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -3949,243 +3762,243 @@
       <c r="N9" s="3"/>
     </row>
     <row r="10" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
-        <v>119</v>
+      <c r="A10" s="19" t="s">
+        <v>88</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>122</v>
+        <v>91</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>117</v>
+        <v>86</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>118</v>
+        <v>87</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>338</v>
+        <v>306</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
     <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="21" t="s">
-        <v>123</v>
+      <c r="A11" s="19" t="s">
+        <v>92</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3" t="s">
-        <v>124</v>
+        <v>93</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>126</v>
+        <v>95</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3" t="s">
-        <v>338</v>
+        <v>306</v>
       </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
     <row r="12" spans="1:15" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="21" t="s">
-        <v>128</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>377</v>
-      </c>
-      <c r="C12" s="10"/>
+      <c r="A12" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="C12" s="9"/>
       <c r="D12" s="3" t="s">
-        <v>363</v>
+        <v>331</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="J12" s="25" t="s">
-        <v>130</v>
+        <v>327</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>99</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>354</v>
+        <v>322</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>353</v>
+        <v>321</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
     <row r="13" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="21" t="s">
-        <v>131</v>
+      <c r="A13" s="19" t="s">
+        <v>100</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>132</v>
+        <v>101</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>133</v>
+        <v>102</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>365</v>
+        <v>333</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>134</v>
+        <v>103</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3" t="s">
-        <v>357</v>
+        <v>325</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>136</v>
+        <v>105</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>338</v>
+        <v>306</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
     <row r="14" spans="1:15" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="21" t="s">
-        <v>137</v>
+      <c r="A14" s="19" t="s">
+        <v>106</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>138</v>
+        <v>107</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>139</v>
+        <v>108</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>364</v>
+        <v>332</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>358</v>
+        <v>326</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>141</v>
+        <v>110</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>136</v>
+        <v>105</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>338</v>
+        <v>306</v>
       </c>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="21" t="s">
-        <v>142</v>
+      <c r="A15" s="19" t="s">
+        <v>111</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>143</v>
+        <v>112</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>144</v>
+        <v>113</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>349</v>
+        <v>317</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J15" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="J15" s="3" t="s">
-        <v>136</v>
-      </c>
       <c r="K15" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
     <row r="16" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>339</v>
+      <c r="A16" s="8" t="s">
+        <v>307</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>340</v>
+        <v>308</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="D16" s="25" t="s">
-        <v>366</v>
+        <v>309</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>334</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>345</v>
+        <v>313</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3" t="s">
-        <v>356</v>
+        <v>324</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>342</v>
+        <v>310</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>342</v>
+        <v>310</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>367</v>
+      <c r="A17" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>335</v>
       </c>
       <c r="C17" s="3"/>
       <c r="F17" s="3"/>
@@ -4199,59 +4012,59 @@
       <c r="N17" s="3"/>
     </row>
     <row r="18" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
-        <v>147</v>
+      <c r="A18" s="19" t="s">
+        <v>116</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>148</v>
+        <v>117</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>368</v>
+        <v>336</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="J18" s="34" t="s">
-        <v>152</v>
+        <v>120</v>
+      </c>
+      <c r="J18" s="32" t="s">
+        <v>121</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
     <row r="19" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="21" t="s">
-        <v>153</v>
+      <c r="A19" s="19" t="s">
+        <v>122</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3" t="s">
-        <v>371</v>
+        <v>339</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>375</v>
+        <v>343</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3" t="s">
-        <v>374</v>
+        <v>342</v>
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
@@ -4261,15 +4074,15 @@
       <c r="N19" s="3"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>156</v>
+      <c r="A20" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>125</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -4282,57 +4095,57 @@
       <c r="N20" s="3"/>
     </row>
     <row r="21" spans="1:14" ht="72" x14ac:dyDescent="0.3">
-      <c r="A21" s="21" t="s">
-        <v>162</v>
+      <c r="A21" s="19" t="s">
+        <v>131</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="E21" s="40" t="s">
-        <v>383</v>
+        <v>350</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>351</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
     <row r="22" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="21" t="s">
-        <v>165</v>
+      <c r="A22" s="19" t="s">
+        <v>134</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>384</v>
+        <v>132</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>352</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="s">
-        <v>164</v>
+        <v>133</v>
       </c>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
@@ -4342,182 +4155,182 @@
       <c r="N22" s="3"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>378</v>
-      </c>
-      <c r="C23" s="10"/>
+      <c r="A23" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="C23" s="9"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
-      <c r="J23" s="25"/>
+      <c r="J23" s="23"/>
       <c r="K23" s="3"/>
-      <c r="L23" s="39"/>
+      <c r="L23" s="36"/>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
     </row>
     <row r="24" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="9"/>
+      <c r="A24" s="8"/>
       <c r="B24" s="3"/>
-      <c r="C24" s="25" t="s">
-        <v>380</v>
+      <c r="C24" s="23" t="s">
+        <v>348</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>167</v>
+        <v>136</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>168</v>
+        <v>137</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="J24" s="25" t="s">
-        <v>169</v>
+        <v>318</v>
+      </c>
+      <c r="J24" s="23" t="s">
+        <v>138</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>352</v>
-      </c>
-      <c r="L24" s="39" t="s">
-        <v>351</v>
+        <v>320</v>
+      </c>
+      <c r="L24" s="36" t="s">
+        <v>319</v>
       </c>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
     </row>
     <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>346</v>
+      <c r="A25" s="8" t="s">
+        <v>314</v>
       </c>
       <c r="B25" s="3"/>
-      <c r="C25" s="39" t="s">
-        <v>348</v>
+      <c r="C25" s="36" t="s">
+        <v>316</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>347</v>
+        <v>315</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3" t="s">
-        <v>355</v>
+        <v>323</v>
       </c>
       <c r="I25" s="3"/>
-      <c r="J25" s="25"/>
+      <c r="J25" s="23"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
     <row r="26" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>379</v>
-      </c>
-      <c r="C26" s="10"/>
+      <c r="A26" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="C26" s="9"/>
       <c r="D26" s="3" t="s">
-        <v>171</v>
+        <v>140</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>172</v>
+        <v>141</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>173</v>
+        <v>142</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>174</v>
+        <v>143</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>176</v>
-      </c>
-      <c r="C27" s="24"/>
+      <c r="A27" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C27" s="22"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3" t="s">
-        <v>177</v>
+        <v>146</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>178</v>
+        <v>147</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>179</v>
+        <v>148</v>
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
     <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="21" t="s">
-        <v>180</v>
+      <c r="A28" s="19" t="s">
+        <v>149</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3" t="s">
-        <v>181</v>
+        <v>150</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I28" s="3"/>
       <c r="N28" s="3"/>
     </row>
     <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="21" t="s">
-        <v>184</v>
+      <c r="A29" s="19" t="s">
+        <v>153</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3" t="s">
-        <v>185</v>
+        <v>154</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>186</v>
+        <v>155</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>187</v>
+        <v>156</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3" t="s">
-        <v>114</v>
+        <v>83</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
@@ -4527,25 +4340,25 @@
       <c r="N29" s="3"/>
     </row>
     <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
-        <v>188</v>
+      <c r="A30" s="19" t="s">
+        <v>157</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3" t="s">
-        <v>189</v>
+        <v>158</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>190</v>
+        <v>159</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>191</v>
+        <v>160</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3" t="s">
-        <v>192</v>
+        <v>161</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
@@ -4555,25 +4368,25 @@
       <c r="N30" s="3"/>
     </row>
     <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="21" t="s">
-        <v>193</v>
+      <c r="A31" s="19" t="s">
+        <v>162</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3" t="s">
-        <v>194</v>
+        <v>163</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>195</v>
+        <v>164</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>196</v>
+        <v>165</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
@@ -4583,105 +4396,105 @@
       <c r="N31" s="3"/>
     </row>
     <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C32" s="10"/>
+      <c r="A32" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="C32" s="9"/>
       <c r="D32" s="3" t="s">
-        <v>199</v>
+        <v>168</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3" t="s">
-        <v>200</v>
+        <v>169</v>
       </c>
       <c r="H32" s="3"/>
       <c r="I32" s="3" t="s">
-        <v>201</v>
+        <v>170</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>202</v>
+        <v>171</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>203</v>
+        <v>172</v>
       </c>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="21" t="s">
-        <v>204</v>
+      <c r="A33" s="19" t="s">
+        <v>173</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="3" t="s">
-        <v>205</v>
+        <v>174</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>206</v>
+        <v>175</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="N33" s="3"/>
     </row>
     <row r="34" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="21" t="s">
-        <v>207</v>
+      <c r="A34" s="19" t="s">
+        <v>176</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3" t="s">
-        <v>208</v>
+        <v>177</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>209</v>
+        <v>178</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="I34" s="3"/>
-      <c r="J34" s="33"/>
+      <c r="J34" s="31"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
     <row r="35" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
-        <v>211</v>
+      <c r="A35" s="8" t="s">
+        <v>180</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3" t="s">
-        <v>372</v>
+        <v>340</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>369</v>
+        <v>337</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3" t="s">
-        <v>370</v>
+        <v>338</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
@@ -4691,26 +4504,26 @@
       <c r="N35" s="3"/>
     </row>
     <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="C36" s="10"/>
+      <c r="A36" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" s="9"/>
       <c r="D36" s="3" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3" t="s">
-        <v>215</v>
+        <v>184</v>
       </c>
       <c r="H36" s="3"/>
       <c r="I36" s="3" t="s">
-        <v>216</v>
+        <v>185</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>217</v>
+        <v>186</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
@@ -4718,53 +4531,53 @@
       <c r="N36" s="3"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="21" t="s">
-        <v>218</v>
+      <c r="A37" s="19" t="s">
+        <v>187</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3" t="s">
-        <v>219</v>
+        <v>188</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>220</v>
+        <v>189</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>221</v>
+        <v>190</v>
       </c>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
     <row r="38" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="21" t="s">
-        <v>222</v>
+      <c r="A38" s="19" t="s">
+        <v>191</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3" t="s">
-        <v>223</v>
+        <v>192</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>224</v>
+        <v>193</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="3" t="s">
-        <v>225</v>
+        <v>194</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
@@ -4774,20 +4587,20 @@
       <c r="N38" s="3"/>
     </row>
     <row r="39" spans="1:14" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="9" t="s">
-        <v>226</v>
+      <c r="A39" s="8" t="s">
+        <v>195</v>
       </c>
       <c r="B39" s="3"/>
-      <c r="C39" s="37" t="s">
-        <v>227</v>
-      </c>
-      <c r="D39" s="27" t="s">
-        <v>228</v>
+      <c r="C39" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="D39" s="25" t="s">
+        <v>197</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
@@ -4797,31 +4610,31 @@
       <c r="N39" s="3"/>
     </row>
     <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="21" t="s">
-        <v>229</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="C40" s="10"/>
+      <c r="A40" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="C40" s="9"/>
       <c r="D40" s="3" t="s">
-        <v>231</v>
+        <v>200</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>168</v>
+        <v>137</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>122</v>
+        <v>91</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="J40" s="22" t="s">
-        <v>233</v>
+        <v>201</v>
+      </c>
+      <c r="J40" s="20" t="s">
+        <v>202</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
@@ -4829,31 +4642,31 @@
       <c r="N40" s="3"/>
     </row>
     <row r="41" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A41" s="21" t="s">
-        <v>234</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="C41" s="10"/>
+      <c r="A41" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="C41" s="9"/>
       <c r="D41" s="3" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>237</v>
+        <v>206</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I41" s="35" t="s">
-        <v>238</v>
-      </c>
-      <c r="J41" s="35" t="s">
-        <v>239</v>
+        <v>79</v>
+      </c>
+      <c r="I41" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="J41" s="33" t="s">
+        <v>208</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
@@ -4861,33 +4674,33 @@
       <c r="N41" s="3"/>
     </row>
     <row r="42" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="21" t="s">
-        <v>240</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="C42" s="10"/>
+      <c r="A42" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="C42" s="9"/>
       <c r="D42" s="3" t="s">
-        <v>242</v>
+        <v>211</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>243</v>
+        <v>212</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>244</v>
+        <v>213</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>245</v>
+        <v>214</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>246</v>
+        <v>215</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
@@ -4895,31 +4708,31 @@
       <c r="N42" s="3"/>
     </row>
     <row r="43" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A43" s="21" t="s">
-        <v>247</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="C43" s="10"/>
+      <c r="A43" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="C43" s="9"/>
       <c r="D43" s="3" t="s">
-        <v>249</v>
+        <v>218</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>250</v>
+        <v>219</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>122</v>
+        <v>91</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>251</v>
+        <v>220</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>252</v>
+        <v>221</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
@@ -4927,22 +4740,22 @@
       <c r="N43" s="3"/>
     </row>
     <row r="44" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A44" s="21" t="s">
-        <v>253</v>
+      <c r="A44" s="19" t="s">
+        <v>222</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="3" t="s">
-        <v>254</v>
+        <v>223</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>255</v>
+        <v>224</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="3" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
@@ -4952,22 +4765,22 @@
       <c r="N44" s="3"/>
     </row>
     <row r="45" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="21" t="s">
-        <v>256</v>
+      <c r="A45" s="19" t="s">
+        <v>225</v>
       </c>
       <c r="B45" s="3"/>
       <c r="C45" s="3" t="s">
-        <v>257</v>
+        <v>226</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>258</v>
+        <v>227</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G45" s="3"/>
       <c r="H45" s="3" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
@@ -4977,31 +4790,31 @@
       <c r="N45" s="3"/>
     </row>
     <row r="46" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A46" s="21" t="s">
-        <v>259</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="C46" s="10"/>
+      <c r="A46" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="C46" s="9"/>
       <c r="D46" s="3" t="s">
-        <v>261</v>
+        <v>230</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>262</v>
+        <v>231</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>122</v>
+        <v>91</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="J46" s="26" t="s">
-        <v>264</v>
+        <v>232</v>
+      </c>
+      <c r="J46" s="24" t="s">
+        <v>233</v>
       </c>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
@@ -5009,111 +4822,111 @@
       <c r="N46" s="3"/>
     </row>
     <row r="47" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>266</v>
-      </c>
-      <c r="C47" s="10"/>
+      <c r="A47" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C47" s="9"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
-      <c r="J47" s="26"/>
+      <c r="J47" s="24"/>
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
     </row>
     <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A48" s="21" t="s">
-        <v>267</v>
-      </c>
-      <c r="B48" s="10"/>
-      <c r="C48" s="22" t="s">
-        <v>268</v>
+      <c r="A48" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="B48" s="9"/>
+      <c r="C48" s="20" t="s">
+        <v>237</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>269</v>
+        <v>238</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>270</v>
+        <v>239</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G48" s="3"/>
       <c r="H48" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="J48" s="22" t="s">
-        <v>272</v>
-      </c>
-      <c r="K48" s="27" t="s">
-        <v>273</v>
-      </c>
-      <c r="L48" s="27"/>
-      <c r="M48" s="27"/>
+        <v>240</v>
+      </c>
+      <c r="J48" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="K48" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="L48" s="25"/>
+      <c r="M48" s="25"/>
       <c r="N48" s="3"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>274</v>
+      <c r="A49" s="8" t="s">
+        <v>243</v>
       </c>
       <c r="B49" s="3"/>
-      <c r="C49" s="22" t="s">
-        <v>275</v>
+      <c r="C49" s="20" t="s">
+        <v>244</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>277</v>
+        <v>245</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>246</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
-      <c r="K49" s="27"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
+      <c r="K49" s="25"/>
+      <c r="L49" s="16"/>
+      <c r="M49" s="16"/>
       <c r="N49" s="3"/>
     </row>
     <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="B50" s="10" t="s">
-        <v>279</v>
-      </c>
-      <c r="C50" s="10"/>
+      <c r="A50" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="C50" s="9"/>
       <c r="D50" s="3" t="s">
-        <v>280</v>
+        <v>249</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>281</v>
+        <v>250</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>122</v>
+        <v>91</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I50" s="35" t="s">
-        <v>282</v>
-      </c>
-      <c r="J50" s="22" t="s">
-        <v>283</v>
+        <v>79</v>
+      </c>
+      <c r="I50" s="33" t="s">
+        <v>251</v>
+      </c>
+      <c r="J50" s="20" t="s">
+        <v>252</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="3"/>
@@ -5121,31 +4934,31 @@
       <c r="N50" s="3"/>
     </row>
     <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A51" s="21" t="s">
-        <v>284</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="C51" s="10"/>
+      <c r="A51" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="C51" s="9"/>
       <c r="D51" s="3" t="s">
-        <v>286</v>
+        <v>255</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>287</v>
+        <v>256</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>288</v>
+        <v>257</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="3" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>289</v>
+        <v>258</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>290</v>
+        <v>259</v>
       </c>
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
@@ -5153,31 +4966,31 @@
       <c r="N51" s="3"/>
     </row>
     <row r="52" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="21" t="s">
-        <v>291</v>
-      </c>
-      <c r="B52" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="C52" s="29"/>
+      <c r="A52" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="B52" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C52" s="27"/>
       <c r="D52" s="3" t="s">
-        <v>292</v>
+        <v>261</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>237</v>
+        <v>206</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="3" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>293</v>
+        <v>262</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>294</v>
+        <v>263</v>
       </c>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
@@ -5185,39 +4998,39 @@
       <c r="N52" s="3"/>
     </row>
     <row r="53" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="9" t="s">
-        <v>295</v>
+      <c r="A53" s="8" t="s">
+        <v>264</v>
       </c>
       <c r="B53" t="s">
-        <v>296</v>
-      </c>
-      <c r="D53" s="23" t="s">
-        <v>297</v>
+        <v>265</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>266</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>298</v>
+        <v>267</v>
       </c>
       <c r="H53" t="s">
-        <v>299</v>
+        <v>268</v>
       </c>
       <c r="I53" t="s">
-        <v>300</v>
+        <v>269</v>
       </c>
       <c r="J53" t="s">
-        <v>301</v>
+        <v>270</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B57" s="30"/>
-      <c r="C57" s="30"/>
+      <c r="B57" s="28"/>
+      <c r="C57" s="28"/>
     </row>
     <row r="58" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="31"/>
-      <c r="C58" s="32"/>
+      <c r="B58" s="29"/>
+      <c r="C58" s="30"/>
     </row>
     <row r="59" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="30"/>
-      <c r="C59" s="30"/>
+      <c r="B59" s="28"/>
+      <c r="C59" s="28"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -5246,48 +5059,48 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>302</v>
+        <v>271</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>303</v>
+        <v>272</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>304</v>
+        <v>273</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>305</v>
+        <v>274</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>306</v>
+        <v>275</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>66</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -5304,7 +5117,7 @@
     <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>307</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -5324,23 +5137,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>308</v>
+        <v>277</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>309</v>
+        <v>278</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>310</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>311</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -5363,61 +5176,61 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="15" t="s">
-        <v>312</v>
-      </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="B2" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="16" t="s">
-        <v>313</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>314</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>315</v>
+      <c r="B3" s="15" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>317</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>318</v>
-      </c>
-      <c r="E4" s="14"/>
+      <c r="B4" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="E4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="14" t="s">
-        <v>319</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>320</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>321</v>
-      </c>
-      <c r="E5" s="14"/>
+      <c r="B5" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="E5" s="13"/>
     </row>
     <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21"/>
+      <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
-        <v>279</v>
+        <v>248</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>323</v>
+        <v>291</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>292</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5426,38 +5239,38 @@
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B7" s="14" t="s">
-        <v>324</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>322</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>325</v>
-      </c>
-      <c r="E7" s="14"/>
+      <c r="B7" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="E7" s="13"/>
     </row>
     <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B8" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="38" t="s">
-        <v>327</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>329</v>
+      <c r="B8" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" s="13"/>
+      <c r="D8" s="35" t="s">
+        <v>295</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="B9" s="14"/>
-      <c r="C9" s="14" t="s">
-        <v>343</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>344</v>
-      </c>
-      <c r="E9" s="25"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="E9" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5468,6 +5281,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -5674,15 +5496,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5695,6 +5508,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5713,14 +5534,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Condition: removed top row of requirements
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichalCiszewski\Documents\Github\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455916BA-1B1A-461D-977E-85F4A305936A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE709FF9-2A2B-4051-BB1C-831A73854CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="2" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -51,7 +51,6 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={FC56F738-FB65-495B-9B48-E0F47216F010}</author>
     <author>tc={903FD87C-9891-4AE1-9361-7224FCD06B01}</author>
     <author>tc={B3533A99-0CB6-4646-9417-20A66FEFD573}</author>
     <author>tc={20B2A504-5F6F-4996-9921-E2104F9548D8}</author>
@@ -61,15 +60,7 @@
     <author>tc={065B39A6-9843-49BF-88E8-0C2BF95F8D00}</author>
   </authors>
   <commentList>
-    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{FC56F738-FB65-495B-9B48-E0F47216F010}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    AllergyInt heeft een andere naam conventie voor ‘Nummer’. Controleren welke juist is.</t>
-      </text>
-    </comment>
-    <comment ref="J21" authorId="1" shapeId="0" xr:uid="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
+    <comment ref="J20" authorId="0" shapeId="0" xr:uid="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -81,7 +72,7 @@
  evolution status - initial, interim/working, final; temporal status - current, past; episodicity status - first, new, ongoing; admission status - admission, discharge; or priority status - primary, secondary.</t>
       </text>
     </comment>
-    <comment ref="K21" authorId="2" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
+    <comment ref="K20" authorId="1" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -91,7 +82,7 @@
 Kortere waardelijst</t>
       </text>
     </comment>
-    <comment ref="K26" authorId="3" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
+    <comment ref="K25" authorId="2" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -99,7 +90,7 @@
     Wel in metadata!</t>
       </text>
     </comment>
-    <comment ref="E29" authorId="4" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
+    <comment ref="E28" authorId="3" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -107,7 +98,7 @@
     Onduidelijk welke waardelijst gehandeerd moet worden</t>
       </text>
     </comment>
-    <comment ref="B31" authorId="5" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
+    <comment ref="B30" authorId="4" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -115,7 +106,7 @@
     ter discussie</t>
       </text>
     </comment>
-    <comment ref="C31" authorId="6" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
+    <comment ref="C30" authorId="5" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -123,7 +114,7 @@
     ter discussie</t>
       </text>
     </comment>
-    <comment ref="C39" authorId="7" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
+    <comment ref="C38" authorId="6" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -136,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="350">
   <si>
     <t>Veld</t>
   </si>
@@ -328,12 +319,6 @@
     <t>Opmerking</t>
   </si>
   <si>
-    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
-  </si>
-  <si>
-    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
-  </si>
-  <si>
     <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
   </si>
   <si>
@@ -341,9 +326,6 @@
   </si>
   <si>
     <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
-  </si>
-  <si>
-    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
   </si>
   <si>
     <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
@@ -1370,7 +1352,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1393,13 +1375,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1610,20 +1585,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1635,27 +1610,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1664,53 +1638,56 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1719,13 +1696,10 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2676,8 +2650,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N53" totalsRowShown="0" headerRowDxfId="12">
-  <autoFilter ref="A2:N53" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N52" totalsRowShown="0" headerRowDxfId="12">
+  <autoFilter ref="A2:N52" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="10"/>
@@ -3039,34 +3013,31 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A3" dT="2026-07-23T07:54:32.60" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{FC56F738-FB65-495B-9B48-E0F47216F010}">
-    <text>AllergyInt heeft een andere naam conventie voor ‘Nummer’. Controleren welke juist is.</text>
-  </threadedComment>
-  <threadedComment ref="J21" dT="2026-07-16T05:50:21.33" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
+  <threadedComment ref="J20" dT="2026-07-16T05:50:21.33" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{903FD87C-9891-4AE1-9361-7224FCD06B01}">
     <text> active
  inactive
  resolved
  in remission
  evolution status - initial, interim/working, final; temporal status - current, past; episodicity status - first, new, ongoing; admission status - admission, discharge; or priority status - primary, secondary.</text>
   </threadedComment>
-  <threadedComment ref="K21" dT="2026-07-20T09:26:12.56" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
+  <threadedComment ref="K20" dT="2026-07-20T09:26:12.56" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
     <text>1. Actief
 2. Inactief
 Kortere waardelijst</text>
   </threadedComment>
-  <threadedComment ref="K26" dT="2026-07-20T09:50:58.06" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
+  <threadedComment ref="K25" dT="2026-07-20T09:50:58.06" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
     <text>Wel in metadata!</text>
   </threadedComment>
-  <threadedComment ref="E29" dT="2026-07-20T11:55:56.61" personId="{86017760-9D2E-4C04-A548-4B0AED173840}" id="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
+  <threadedComment ref="E28" dT="2026-07-20T11:55:56.61" personId="{86017760-9D2E-4C04-A548-4B0AED173840}" id="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
     <text>Onduidelijk welke waardelijst gehandeerd moet worden</text>
   </threadedComment>
-  <threadedComment ref="B31" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
+  <threadedComment ref="B30" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
     <text>ter discussie</text>
   </threadedComment>
-  <threadedComment ref="C31" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
+  <threadedComment ref="C30" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
     <text>ter discussie</text>
   </threadedComment>
-  <threadedComment ref="C39" dT="2026-07-22T10:57:31.61" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
+  <threadedComment ref="C38" dT="2026-07-22T10:57:31.61" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
     <text>ter discussie</text>
   </threadedComment>
 </ThreadedComments>
@@ -3131,143 +3102,143 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="40"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
     </row>
     <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="40"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="39"/>
     </row>
     <row r="5" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="40"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="39"/>
     </row>
     <row r="6" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="40"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="39"/>
     </row>
     <row r="7" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="41"/>
+      <c r="D7" s="40"/>
     </row>
     <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="42"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="41"/>
     </row>
     <row r="9" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="41"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="40"/>
     </row>
     <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="40"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="39"/>
     </row>
     <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>298</v>
-      </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="40"/>
+        <v>295</v>
+      </c>
+      <c r="C11" s="38"/>
+      <c r="D11" s="39"/>
     </row>
     <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C12" s="39"/>
-      <c r="D12" s="40"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="39"/>
     </row>
     <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B13" s="43"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="40"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="39"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B14" s="5"/>
-      <c r="C14" s="44"/>
+      <c r="C14" s="43"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
-      <c r="C15" s="44"/>
+      <c r="C15" s="43"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="43"/>
-      <c r="C16" s="44"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="43"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="43"/>
-      <c r="C17" s="44"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="43"/>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="43"/>
-      <c r="C18" s="39"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="38"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="43"/>
-      <c r="C19" s="44"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="43"/>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="43"/>
-      <c r="C20" s="44"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="43"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="39"/>
-      <c r="C21" s="44"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="43"/>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B22" s="43"/>
-      <c r="C22" s="44"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="43"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B23" s="43"/>
-      <c r="C23" s="44"/>
+      <c r="B23" s="42"/>
+      <c r="C23" s="43"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B24" s="43"/>
-      <c r="C24" s="39"/>
+      <c r="B24" s="42"/>
+      <c r="C24" s="38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3318,7 +3289,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -3431,7 +3402,7 @@
         <v>28</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -3511,7 +3482,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
@@ -3574,80 +3545,84 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="71.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>63</v>
+    <row r="3" spans="1:15" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>67</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C3" s="17"/>
-      <c r="D3" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H3" s="1" t="s">
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="3" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+      <c r="J3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="3" t="s">
+      <c r="K3" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="L3" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="N3" s="18"/>
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="C4" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="K4" s="19" t="s">
-        <v>305</v>
-      </c>
-      <c r="L4" s="19" t="s">
-        <v>305</v>
-      </c>
-      <c r="M4" s="19" t="s">
-        <v>305</v>
-      </c>
-      <c r="N4" s="19"/>
-      <c r="O4" s="8"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="D4" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>75</v>
       </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="7"/>
       <c r="C5" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -3656,26 +3631,26 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
-        <v>80</v>
+    <row r="6" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>298</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -3684,26 +3659,26 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="19" t="s">
-        <v>84</v>
+    <row r="7" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>301</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7" t="s">
-        <v>76</v>
+        <v>274</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>303</v>
+        <v>326</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>301</v>
+        <v>74</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>29</v>
+        <v>325</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -3712,27 +3687,20 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>304</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7" t="s">
-        <v>277</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" s="7"/>
       <c r="D8" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>78</v>
-      </c>
+        <v>327</v>
+      </c>
+      <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3" t="s">
-        <v>328</v>
-      </c>
+      <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
@@ -3740,332 +3708,332 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="26" t="s">
-        <v>299</v>
-      </c>
-      <c r="C9" s="7"/>
+      <c r="C9" s="3" t="s">
+        <v>86</v>
+      </c>
       <c r="D9" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="F9" s="3"/>
+        <v>87</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>303</v>
+      </c>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="19" t="s">
-        <v>88</v>
-      </c>
+    <row r="10" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>74</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
       <c r="L10" s="3" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3" t="s">
-        <v>93</v>
-      </c>
+    <row r="11" spans="1:15" ht="72" x14ac:dyDescent="0.3">
+      <c r="A11" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="C11" s="9"/>
       <c r="D11" s="3" t="s">
-        <v>94</v>
+        <v>328</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>95</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="J11" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+      <c r="K11" s="3" t="s">
+        <v>319</v>
+      </c>
       <c r="L11" s="3" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:15" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+    <row r="12" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>345</v>
-      </c>
-      <c r="C12" s="9"/>
+      <c r="B12" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="D12" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>98</v>
-      </c>
+        <v>330</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>79</v>
+        <v>322</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>322</v>
+        <v>71</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="19" t="s">
-        <v>100</v>
+    <row r="13" spans="1:15" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="18" t="s">
+        <v>103</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:15" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="19" t="s">
-        <v>106</v>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" s="18" t="s">
+        <v>108</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>332</v>
+        <v>314</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>326</v>
+        <v>76</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>110</v>
+        <v>71</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>306</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
-        <v>111</v>
+    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>304</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>112</v>
+        <v>305</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>317</v>
+        <v>306</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>331</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>114</v>
+        <v>310</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3" t="s">
-        <v>79</v>
+        <v>321</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>74</v>
+        <v>307</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>105</v>
+        <v>307</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>307</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>334</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>313</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="C16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B17" s="22" t="s">
-        <v>335</v>
-      </c>
-      <c r="C17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="F17" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="J17" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
-        <v>116</v>
+    <row r="18" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>117</v>
+        <v>336</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>118</v>
+        <v>338</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="J18" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>74</v>
-      </c>
+        <v>339</v>
+      </c>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="19" t="s">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3" t="s">
-        <v>339</v>
-      </c>
+      <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>78</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="3" t="s">
-        <v>342</v>
-      </c>
+      <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
@@ -4073,264 +4041,271 @@
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
+    <row r="20" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A20" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="D20" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="E20" s="36" t="s">
+        <v>348</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3" t="s">
+      <c r="J20" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
+      <c r="K20" s="3" t="s">
+        <v>127</v>
+      </c>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
     </row>
-    <row r="21" spans="1:14" ht="72" x14ac:dyDescent="0.3">
-      <c r="A21" s="19" t="s">
+    <row r="21" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="18" t="s">
         <v>131</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="E21" s="37" t="s">
-        <v>351</v>
+        <v>129</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>349</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="K21" s="3" t="s">
         <v>130</v>
       </c>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="D22" s="3" t="s">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="E22" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>78</v>
-      </c>
+      <c r="B22" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="C22" s="9"/>
+      <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="3" t="s">
-        <v>133</v>
-      </c>
+      <c r="H22" s="3"/>
       <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
+      <c r="J22" s="22"/>
       <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
+      <c r="L22" s="35"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="19" t="s">
+    <row r="23" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="8"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="22" t="s">
+        <v>345</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="J23" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>346</v>
-      </c>
-      <c r="C23" s="9"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="36"/>
+      <c r="K23" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="L23" s="35" t="s">
+        <v>316</v>
+      </c>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
     </row>
     <row r="24" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="8"/>
+      <c r="A24" s="8" t="s">
+        <v>311</v>
+      </c>
       <c r="B24" s="3"/>
-      <c r="C24" s="23" t="s">
-        <v>348</v>
+      <c r="C24" s="35" t="s">
+        <v>313</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>119</v>
-      </c>
+        <v>312</v>
+      </c>
+      <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="J24" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="K24" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="L24" s="36" t="s">
-        <v>319</v>
-      </c>
+      <c r="I24" s="3"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
     </row>
-    <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
-        <v>314</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="36" t="s">
-        <v>316</v>
-      </c>
+    <row r="25" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="C25" s="9"/>
       <c r="D25" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="F25" s="3"/>
+        <v>137</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="I25" s="3"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="3"/>
+        <v>76</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
-    <row r="26" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>347</v>
-      </c>
-      <c r="C26" s="9"/>
-      <c r="D26" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E26" s="3" t="s">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="F26" s="3" t="s">
-        <v>119</v>
-      </c>
+      <c r="B26" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="F26" s="3"/>
       <c r="G26" s="3"/>
-      <c r="H26" s="3" t="s">
-        <v>79</v>
-      </c>
+      <c r="H26" s="3"/>
       <c r="I26" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>74</v>
+        <v>145</v>
       </c>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="C27" s="22"/>
-      <c r="F27" s="3"/>
+    <row r="27" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
+      <c r="H27" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="19" t="s">
-        <v>149</v>
+    <row r="28" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="18" t="s">
+        <v>150</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="19" t="s">
-        <v>153</v>
+    <row r="29" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="18" t="s">
+        <v>154</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3" t="s">
-        <v>83</v>
+        <v>158</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
@@ -4339,26 +4314,26 @@
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="19" t="s">
-        <v>157</v>
+    <row r="30" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="18" t="s">
+        <v>159</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>78</v>
+        <v>116</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3" t="s">
-        <v>161</v>
+        <v>93</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
@@ -4367,65 +4342,60 @@
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3" t="s">
+    <row r="31" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
         <v>163</v>
       </c>
+      <c r="B31" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C31" s="9"/>
       <c r="D31" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="E31" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="F31" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>169</v>
+      </c>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
     </row>
-    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="C32" s="9"/>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3" t="s">
+        <v>171</v>
+      </c>
       <c r="D32" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="K32" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
+      <c r="E32" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
+    <row r="33" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
         <v>173</v>
       </c>
       <c r="B33" s="3"/>
@@ -4436,148 +4406,148 @@
         <v>175</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3" t="s">
-        <v>79</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="I33" s="3"/>
+      <c r="J33" s="30"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="19" t="s">
-        <v>176</v>
+    <row r="34" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3" t="s">
-        <v>177</v>
+        <v>337</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>178</v>
+        <v>334</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>123</v>
+        <v>338</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3" t="s">
-        <v>179</v>
+        <v>335</v>
       </c>
       <c r="I34" s="3"/>
-      <c r="J34" s="31"/>
+      <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>183</v>
+      </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="C36" s="9"/>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="D36" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="J36" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="K36" s="3"/>
+      <c r="E36" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>187</v>
+      </c>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="19" t="s">
-        <v>187</v>
+    <row r="37" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="18" t="s">
+        <v>188</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="K37" s="3" t="s">
-        <v>190</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="19" t="s">
-        <v>191</v>
+    <row r="38" spans="1:14" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
+        <v>192</v>
       </c>
       <c r="B38" s="3"/>
-      <c r="C38" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D38" s="3" t="s">
+      <c r="C38" s="33" t="s">
         <v>193</v>
       </c>
-      <c r="E38" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>119</v>
-      </c>
+      <c r="D38" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3" t="s">
-        <v>194</v>
+        <v>93</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
@@ -4586,121 +4556,130 @@
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
+    <row r="39" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="B39" s="3"/>
-      <c r="C39" s="34" t="s">
+      <c r="B39" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="D39" s="25" t="s">
+      <c r="C39" s="9"/>
+      <c r="D39" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="F39" s="3"/>
+      <c r="E39" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
+        <v>76</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="J39" s="19" t="s">
+        <v>199</v>
+      </c>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="19" t="s">
-        <v>198</v>
+    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="18" t="s">
+        <v>200</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>137</v>
+        <v>203</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="J40" s="20" t="s">
-        <v>202</v>
+        <v>76</v>
+      </c>
+      <c r="I40" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="J40" s="32" t="s">
+        <v>205</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A41" s="19" t="s">
-        <v>203</v>
+    <row r="41" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="18" t="s">
+        <v>206</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G41" s="3"/>
+        <v>116</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>210</v>
+      </c>
       <c r="H41" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I41" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="J41" s="33" t="s">
-        <v>208</v>
+        <v>76</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>212</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="19" t="s">
-        <v>209</v>
+    <row r="42" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="18" t="s">
+        <v>213</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>213</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="G42" s="3"/>
       <c r="H42" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
@@ -4708,39 +4687,32 @@
       <c r="N42" s="3"/>
     </row>
     <row r="43" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A43" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="C43" s="9"/>
+      <c r="A43" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3" t="s">
+        <v>220</v>
+      </c>
       <c r="D43" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="J43" s="3" t="s">
-        <v>221</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
     </row>
     <row r="44" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="18" t="s">
         <v>222</v>
       </c>
       <c r="B44" s="3"/>
@@ -4751,11 +4723,11 @@
         <v>224</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
@@ -4764,276 +4736,251 @@
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="19" t="s">
+    <row r="45" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3" t="s">
+      <c r="B45" s="9" t="s">
         <v>226</v>
       </c>
+      <c r="C45" s="9"/>
       <c r="D45" s="3" t="s">
         <v>227</v>
       </c>
+      <c r="E45" s="3" t="s">
+        <v>228</v>
+      </c>
       <c r="F45" s="3" t="s">
-        <v>119</v>
+        <v>88</v>
       </c>
       <c r="G45" s="3"/>
       <c r="H45" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="I45" s="3"/>
-      <c r="J45" s="3"/>
+        <v>76</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="J45" s="23" t="s">
+        <v>230</v>
+      </c>
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A46" s="19" t="s">
-        <v>228</v>
+    <row r="46" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="8" t="s">
+        <v>231</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C46" s="9"/>
-      <c r="D46" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>91</v>
-      </c>
+      <c r="F46" s="3"/>
       <c r="G46" s="3"/>
-      <c r="H46" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I46" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="J46" s="24" t="s">
-        <v>233</v>
-      </c>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="23"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
     <row r="47" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="8" t="s">
+      <c r="A47" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="B47" s="9"/>
+      <c r="C47" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="D47" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="C47" s="9"/>
-      <c r="F47" s="3"/>
+      <c r="E47" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-      <c r="J47" s="24"/>
-      <c r="K47" s="3"/>
-      <c r="L47" s="3"/>
-      <c r="M47" s="3"/>
+      <c r="H47" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J47" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="K47" s="24" t="s">
+        <v>239</v>
+      </c>
+      <c r="L47" s="24"/>
+      <c r="M47" s="24"/>
       <c r="N47" s="3"/>
     </row>
-    <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A48" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="B48" s="9"/>
-      <c r="C48" s="20" t="s">
-        <v>237</v>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="19" t="s">
+        <v>241</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>243</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G48" s="3"/>
       <c r="H48" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I48" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="J48" s="20" t="s">
-        <v>241</v>
-      </c>
-      <c r="K48" s="25" t="s">
-        <v>242</v>
-      </c>
-      <c r="L48" s="25"/>
-      <c r="M48" s="25"/>
+        <v>176</v>
+      </c>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="24"/>
+      <c r="L48" s="16"/>
+      <c r="M48" s="16"/>
       <c r="N48" s="3"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="B49" s="3"/>
-      <c r="C49" s="20" t="s">
+    <row r="49" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="18" t="s">
         <v>244</v>
       </c>
+      <c r="B49" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="C49" s="9"/>
       <c r="D49" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="E49" s="9" t="s">
         <v>246</v>
       </c>
+      <c r="E49" s="3" t="s">
+        <v>247</v>
+      </c>
       <c r="F49" s="3" t="s">
-        <v>119</v>
+        <v>88</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
-      <c r="K49" s="25"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
+        <v>76</v>
+      </c>
+      <c r="I49" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="J49" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
       <c r="N49" s="3"/>
     </row>
     <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="19" t="s">
-        <v>247</v>
+      <c r="A50" s="18" t="s">
+        <v>250</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>91</v>
+        <v>254</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I50" s="33" t="s">
-        <v>251</v>
-      </c>
-      <c r="J50" s="20" t="s">
-        <v>252</v>
+        <v>76</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>256</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="3"/>
       <c r="M50" s="3"/>
       <c r="N50" s="3"/>
     </row>
-    <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A51" s="19" t="s">
-        <v>253</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="C51" s="9"/>
+    <row r="51" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="B51" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C51" s="26"/>
       <c r="D51" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>256</v>
+        <v>203</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>257</v>
+        <v>116</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="3" t="s">
-        <v>79</v>
+        <v>176</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
       <c r="N51" s="3"/>
     </row>
-    <row r="52" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="19" t="s">
-        <v>260</v>
-      </c>
-      <c r="B52" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="C52" s="27"/>
-      <c r="D52" s="3" t="s">
+    <row r="52" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="8" t="s">
         <v>261</v>
       </c>
+      <c r="B52" t="s">
+        <v>262</v>
+      </c>
+      <c r="D52" s="20" t="s">
+        <v>263</v>
+      </c>
       <c r="E52" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="J52" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="K52" s="3"/>
-      <c r="L52" s="3"/>
-      <c r="M52" s="3"/>
-      <c r="N52" s="3"/>
-    </row>
-    <row r="53" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="B53" t="s">
+      <c r="H52" t="s">
         <v>265</v>
       </c>
-      <c r="D53" s="21" t="s">
+      <c r="I52" t="s">
         <v>266</v>
       </c>
-      <c r="E53" s="3" t="s">
+      <c r="J52" t="s">
         <v>267</v>
       </c>
-      <c r="H53" t="s">
-        <v>268</v>
-      </c>
-      <c r="I53" t="s">
-        <v>269</v>
-      </c>
-      <c r="J53" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B56" s="27"/>
+      <c r="C56" s="27"/>
+    </row>
+    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="28"/>
-      <c r="C57" s="28"/>
-    </row>
-    <row r="58" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="29"/>
-      <c r="C58" s="30"/>
-    </row>
-    <row r="59" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="28"/>
-      <c r="C59" s="28"/>
+      <c r="C57" s="29"/>
+    </row>
+    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="27"/>
+      <c r="C58" s="27"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -5059,10 +5006,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>50</v>
@@ -5082,25 +5029,25 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -5117,7 +5064,7 @@
     <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -5137,7 +5084,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B1" t="s">
         <v>22</v>
@@ -5145,15 +5092,15 @@
     </row>
     <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -5177,7 +5124,7 @@
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -5185,52 +5132,52 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C3" s="15" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="13" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E4" s="13"/>
     </row>
     <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="18"/>
+      <c r="B6" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D6" s="19" t="s">
         <v>289</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>290</v>
-      </c>
-      <c r="E5" s="13"/>
-    </row>
-    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="19"/>
-      <c r="B6" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>292</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5240,37 +5187,37 @@
     </row>
     <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="13" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C7" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>291</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>294</v>
       </c>
       <c r="E7" s="13"/>
     </row>
     <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C8" s="13"/>
-      <c r="D8" s="35" t="s">
-        <v>295</v>
+      <c r="D8" s="34" t="s">
+        <v>292</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B9" s="13"/>
       <c r="C9" s="13" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="E9" s="23"/>
+        <v>309</v>
+      </c>
+      <c r="E9" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5281,12 +5228,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5497,20 +5446,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5535,12 +5485,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Condition: removed explanation row from requirements file
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl-my.sharepoint.com/personal/eduard_derijcke_nictiz_nl/Documents/Bureaublad/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Nictiz\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8B207D1-1355-40B1-8598-1BBE603C0CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD10C5A-4E46-4677-812B-8C2FB5410E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -63,7 +63,6 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={FC56F738-FB65-495B-9B48-E0F47216F010}</author>
     <author>tc={B3533A99-0CB6-4646-9417-20A66FEFD573}</author>
     <author>tc={20B2A504-5F6F-4996-9921-E2104F9548D8}</author>
     <author>tc={DC3A08E9-01DD-48D1-B7F5-357810DE5428}</author>
@@ -72,15 +71,7 @@
     <author>tc={065B39A6-9843-49BF-88E8-0C2BF95F8D00}</author>
   </authors>
   <commentList>
-    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{FC56F738-FB65-495B-9B48-E0F47216F010}">
-      <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
-    AllergyInt heeft een andere naam conventie voor ‘Nummer’. Controleren welke juist is.</t>
-      </text>
-    </comment>
-    <comment ref="K21" authorId="1" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
+    <comment ref="K20" authorId="0" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -90,7 +81,7 @@
 Kortere waardelijst</t>
       </text>
     </comment>
-    <comment ref="K27" authorId="2" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
+    <comment ref="K26" authorId="1" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -98,7 +89,7 @@
     Wel in metadata!</t>
       </text>
     </comment>
-    <comment ref="E30" authorId="3" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
+    <comment ref="E29" authorId="2" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -106,7 +97,7 @@
     Onduidelijk welke waardelijst gehandeerd moet worden</t>
       </text>
     </comment>
-    <comment ref="B32" authorId="4" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
+    <comment ref="B31" authorId="3" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -114,7 +105,7 @@
     ter discussie</t>
       </text>
     </comment>
-    <comment ref="C32" authorId="5" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
+    <comment ref="C31" authorId="4" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -122,7 +113,7 @@
     ter discussie</t>
       </text>
     </comment>
-    <comment ref="C40" authorId="6" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
+    <comment ref="C39" authorId="5" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
@@ -135,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="391">
   <si>
     <t>Veld</t>
   </si>
@@ -375,12 +366,6 @@
     <t>Opmerking</t>
   </si>
   <si>
-    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
-  </si>
-  <si>
-    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
-  </si>
-  <si>
     <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
   </si>
   <si>
@@ -388,9 +373,6 @@
   </si>
   <si>
     <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
-  </si>
-  <si>
-    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
   </si>
   <si>
     <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
@@ -1592,7 +1574,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1615,13 +1597,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1812,20 +1787,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1840,27 +1815,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1869,53 +1843,53 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2863,8 +2837,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N60" totalsRowShown="0" headerRowDxfId="12">
-  <autoFilter ref="A2:N60" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N59" totalsRowShown="0" headerRowDxfId="12">
+  <autoFilter ref="A2:N59" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="10"/>
@@ -3234,27 +3208,24 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A3" dT="2026-07-23T07:54:32.60" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{FC56F738-FB65-495B-9B48-E0F47216F010}">
-    <text>AllergyInt heeft een andere naam conventie voor ‘Nummer’. Controleren welke juist is.</text>
-  </threadedComment>
-  <threadedComment ref="K21" dT="2026-07-20T09:26:12.56" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
+  <threadedComment ref="K20" dT="2026-07-20T09:26:12.56" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
     <text>1. Actief
 2. Inactief
 Kortere waardelijst</text>
   </threadedComment>
-  <threadedComment ref="K27" dT="2026-07-20T09:50:58.06" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
+  <threadedComment ref="K26" dT="2026-07-20T09:50:58.06" personId="{E6DC4CC4-5331-4633-9C1C-269F406E61BD}" id="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
     <text>Wel in metadata!</text>
   </threadedComment>
-  <threadedComment ref="E30" dT="2026-07-20T11:55:56.61" personId="{86017760-9D2E-4C04-A548-4B0AED173840}" id="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
+  <threadedComment ref="E29" dT="2026-07-20T11:55:56.61" personId="{86017760-9D2E-4C04-A548-4B0AED173840}" id="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
     <text>Onduidelijk welke waardelijst gehandeerd moet worden</text>
   </threadedComment>
-  <threadedComment ref="B32" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
+  <threadedComment ref="B31" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
     <text>ter discussie</text>
   </threadedComment>
-  <threadedComment ref="C32" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
+  <threadedComment ref="C31" dT="2026-07-22T10:46:13.79" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
     <text>ter discussie</text>
   </threadedComment>
-  <threadedComment ref="C40" dT="2026-07-22T10:57:31.61" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
+  <threadedComment ref="C39" dT="2026-07-22T10:57:31.61" personId="{67CE0BAC-4786-48DE-9DCD-69E1F3FACFC1}" id="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
     <text>ter discussie</text>
   </threadedComment>
 </ThreadedComments>
@@ -3424,7 +3395,7 @@
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="3" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3682,7 +3653,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -3745,80 +3716,84 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>77</v>
+    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C3" s="18"/>
-      <c r="D3" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H3" s="1" t="s">
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
+      <c r="J3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="K3" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="3" t="s">
+      <c r="L3" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="M3" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="N3" s="19"/>
+      <c r="O3" s="9"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="C4" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="20" t="s">
+      <c r="D4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="L4" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="M4" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="N4" s="20"/>
-      <c r="O4" s="9"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="E4" s="3" t="s">
         <v>89</v>
       </c>
+      <c r="F4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>93</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -3827,26 +3802,26 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
-        <v>95</v>
+    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
+        <v>97</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>99</v>
+        <v>42</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -3855,26 +3830,26 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+    <row r="7" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>100</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>93</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -3883,27 +3858,20 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8" t="s">
         <v>104</v>
       </c>
+      <c r="B8" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="8"/>
       <c r="D8" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>93</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3" t="s">
-        <v>106</v>
-      </c>
+      <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
@@ -3911,332 +3879,332 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+    <row r="9" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="C9" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C9" s="8"/>
       <c r="D9" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
-        <v>110</v>
-      </c>
+    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I10" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3" t="s">
-        <v>119</v>
-      </c>
+    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C11" s="10"/>
       <c r="D11" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="J11" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>126</v>
+      </c>
       <c r="L11" s="3" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="C12" s="10"/>
+    <row r="12" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>130</v>
+      </c>
       <c r="D12" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>126</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J12" s="24" t="s">
-        <v>128</v>
+        <v>134</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="105" x14ac:dyDescent="0.25">
-      <c r="A13" s="20" t="s">
-        <v>131</v>
+    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>136</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
-        <v>139</v>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
+        <v>143</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>117</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="20" t="s">
-        <v>146</v>
+    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>148</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>151</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3" t="s">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>116</v>
+        <v>154</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>154</v>
-      </c>
-      <c r="E16" s="3" t="s">
         <v>155</v>
       </c>
+      <c r="B16" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>116</v>
-      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="D17" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="J17" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="20" t="s">
-        <v>160</v>
+    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
+        <v>164</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>164</v>
+        <v>90</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="J18" s="33" t="s">
-        <v>166</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>116</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="20" t="s">
-        <v>167</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3" t="s">
-        <v>168</v>
-      </c>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>93</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="3" t="s">
-        <v>171</v>
-      </c>
+      <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
@@ -4244,309 +4212,319 @@
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C20" s="3"/>
       <c r="D20" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="F20" s="3"/>
+      <c r="E20" s="37" t="s">
+        <v>175</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
+      <c r="H20" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="J20" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-    </row>
-    <row r="21" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
-        <v>175</v>
+      <c r="N20" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
+        <v>180</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E21" s="38" t="s">
-        <v>178</v>
+        <v>181</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>182</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>94</v>
+        <v>183</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="J21" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>181</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
-      <c r="N21" s="4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D22" s="3" t="s">
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="B22" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>93</v>
-      </c>
+      <c r="C22" s="10"/>
+      <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>138</v>
-      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="23"/>
       <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
+      <c r="L22" s="36"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="20" t="s">
+    <row r="23" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="D23" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="F23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="37"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-    </row>
-    <row r="24" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="H23" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="J23" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="L23" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="N23" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B24" s="3"/>
-      <c r="C24" s="24" t="s">
-        <v>190</v>
+      <c r="C24" s="23" t="s">
+        <v>197</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I24" s="39" t="s">
-        <v>193</v>
-      </c>
-      <c r="J24" s="24" t="s">
-        <v>194</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="L24" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="M24" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="N24" s="5" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="I24" s="38"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="39"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="5"/>
+    </row>
+    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B25" s="3"/>
-      <c r="C25" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="D25" s="3" t="s">
+      <c r="C25" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="D25" s="37" t="s">
         <v>202</v>
       </c>
+      <c r="E25" s="37" t="s">
+        <v>203</v>
+      </c>
       <c r="F25" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="I25" s="39"/>
-      <c r="J25" s="24"/>
+        <v>204</v>
+      </c>
+      <c r="I25" s="3"/>
+      <c r="J25" s="23"/>
       <c r="K25" s="3"/>
-      <c r="L25" s="40"/>
+      <c r="L25" s="3"/>
       <c r="M25" s="3"/>
-      <c r="N25" s="5"/>
-    </row>
-    <row r="26" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="37" t="s">
-        <v>204</v>
-      </c>
-      <c r="D26" s="38" t="s">
+      <c r="N25" s="3"/>
+    </row>
+    <row r="26" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="E26" s="38" t="s">
+      <c r="B26" s="10" t="s">
         <v>206</v>
       </c>
+      <c r="C26" s="10"/>
+      <c r="D26" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>208</v>
+      </c>
       <c r="F26" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="I26" s="3"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="C27" s="10"/>
-      <c r="D27" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="E27" s="3" t="s">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>164</v>
-      </c>
+      <c r="B27" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C27" s="22"/>
+      <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="3" t="s">
-        <v>94</v>
-      </c>
+      <c r="H27" s="3"/>
       <c r="I27" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>116</v>
+        <v>215</v>
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="B28" s="23" t="s">
-        <v>215</v>
-      </c>
-      <c r="C28" s="23"/>
-      <c r="F28" s="3"/>
+    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
+      <c r="H28" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I28" s="3"/>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
-        <v>219</v>
+    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="19" t="s">
+        <v>220</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="s">
-        <v>223</v>
+    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="19" t="s">
+        <v>224</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3" t="s">
-        <v>99</v>
+        <v>228</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
@@ -4555,26 +4533,26 @@
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="20" t="s">
-        <v>227</v>
+    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="19" t="s">
+        <v>229</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>93</v>
+        <v>161</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
@@ -4583,65 +4561,60 @@
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
     </row>
-    <row r="32" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3" t="s">
-        <v>233</v>
-      </c>
+    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="C32" s="10"/>
       <c r="D32" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>240</v>
+      </c>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="C33" s="10"/>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3" t="s">
+        <v>242</v>
+      </c>
       <c r="D33" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="K33" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
+      <c r="E33" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="20" t="s">
+    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
         <v>244</v>
       </c>
       <c r="B34" s="3"/>
@@ -4652,148 +4625,153 @@
         <v>246</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>163</v>
+        <v>247</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3" t="s">
-        <v>94</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="I34" s="3"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="20" t="s">
-        <v>247</v>
+    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>249</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>164</v>
+        <v>90</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="I35" s="3"/>
-      <c r="J35" s="32"/>
+      <c r="J35" s="3"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3" t="s">
-        <v>253</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="C36" s="10"/>
       <c r="D36" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>259</v>
+      </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="C37" s="10"/>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="D37" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="J37" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="K37" s="3"/>
+      <c r="E37" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>263</v>
+      </c>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="20" t="s">
-        <v>263</v>
+    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
+        <v>264</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>163</v>
+        <v>267</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>266</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="20" t="s">
-        <v>267</v>
+    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>268</v>
       </c>
       <c r="B39" s="3"/>
-      <c r="C39" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="D39" s="3" t="s">
+      <c r="C39" s="34" t="s">
         <v>269</v>
       </c>
+      <c r="D39" s="17" t="s">
+        <v>270</v>
+      </c>
       <c r="E39" s="3" t="s">
-        <v>270</v>
+        <v>160</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3" t="s">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
@@ -4802,217 +4780,217 @@
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="B40" s="3"/>
-      <c r="C40" s="35" t="s">
+    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="B40" s="10" t="s">
         <v>273</v>
       </c>
+      <c r="C40" s="10"/>
+      <c r="D40" s="3" t="s">
+        <v>274</v>
+      </c>
       <c r="E40" s="3" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="J40" s="20" t="s">
+        <v>276</v>
+      </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="20" t="s">
-        <v>275</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>276</v>
-      </c>
+    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="B41" s="3"/>
       <c r="C41" s="10"/>
       <c r="D41" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>192</v>
+        <v>279</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>113</v>
+        <v>161</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="3" t="s">
-        <v>94</v>
+        <v>280</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="J41" s="21" t="s">
-        <v>279</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B42" s="3"/>
       <c r="C42" s="10"/>
       <c r="D42" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="J42" s="3"/>
+        <v>284</v>
+      </c>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3" t="s">
+        <v>285</v>
+      </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
     </row>
-    <row r="43" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="B43" s="3"/>
+    <row r="43" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>287</v>
+      </c>
       <c r="C43" s="10"/>
       <c r="D43" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="I43" s="3"/>
-      <c r="J43" s="3" t="s">
-        <v>288</v>
+        <v>91</v>
+      </c>
+      <c r="I43" s="33" t="s">
+        <v>290</v>
+      </c>
+      <c r="J43" s="33" t="s">
+        <v>291</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
     </row>
-    <row r="44" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="20" t="s">
-        <v>289</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>290</v>
-      </c>
+    <row r="44" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" s="3"/>
       <c r="C44" s="10"/>
       <c r="D44" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="E44" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="F44" s="3" t="s">
-        <v>164</v>
-      </c>
+      <c r="F44" s="3"/>
       <c r="G44" s="3"/>
-      <c r="H44" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I44" s="34" t="s">
-        <v>293</v>
-      </c>
-      <c r="J44" s="34" t="s">
-        <v>294</v>
-      </c>
+      <c r="H44" s="3"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A45" s="9"/>
-      <c r="B45" s="3"/>
+    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>294</v>
+      </c>
       <c r="C45" s="10"/>
       <c r="D45" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
-      <c r="I45" s="34"/>
-      <c r="J45" s="34"/>
+      <c r="E45" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>299</v>
+      </c>
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="20" t="s">
-        <v>296</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>297</v>
-      </c>
+    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="B46" s="3"/>
       <c r="C46" s="10"/>
       <c r="D46" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I46" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="J46" s="3" t="s">
-        <v>302</v>
-      </c>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
-    <row r="47" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="B47" s="3"/>
-      <c r="C47" s="10"/>
       <c r="D47" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="F47" s="3"/>
+      <c r="E47" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="F47" s="3">
+        <v>1</v>
+      </c>
       <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
+      <c r="H47" s="3" t="s">
+        <v>284</v>
+      </c>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
@@ -5020,68 +4998,65 @@
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
     </row>
-    <row r="48" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3" t="s">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" s="19" t="s">
         <v>306</v>
       </c>
+      <c r="B48" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="C48" s="10"/>
       <c r="D48" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="F48" s="3">
-        <v>1</v>
+        <v>309</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>110</v>
       </c>
       <c r="G48" s="3"/>
       <c r="H48" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="I48" s="3"/>
-      <c r="J48" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>311</v>
+      </c>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="20" t="s">
-        <v>309</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>310</v>
-      </c>
-      <c r="C49" s="10"/>
+      <c r="A49" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3" t="s">
+        <v>313</v>
+      </c>
       <c r="D49" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>113</v>
+        <v>161</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I49" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="J49" s="3" t="s">
-        <v>314</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="20" t="s">
+    <row r="50" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="19" t="s">
         <v>315</v>
       </c>
       <c r="B50" s="3"/>
@@ -5092,11 +5067,11 @@
         <v>317</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I50" s="3"/>
       <c r="J50" s="3"/>
@@ -5106,298 +5081,273 @@
       <c r="N50" s="3"/>
     </row>
     <row r="51" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="20" t="s">
+      <c r="A51" s="19" t="s">
         <v>318</v>
       </c>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3" t="s">
+      <c r="B51" s="10" t="s">
         <v>319</v>
       </c>
+      <c r="C51" s="10"/>
       <c r="D51" s="3" t="s">
         <v>320</v>
       </c>
+      <c r="E51" s="3" t="s">
+        <v>321</v>
+      </c>
       <c r="F51" s="3" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="I51" s="3"/>
-      <c r="J51" s="3"/>
-      <c r="K51" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="J51" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="K51" s="4"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
-      <c r="N51" s="3"/>
+      <c r="N51" s="4" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A52" s="20" t="s">
-        <v>321</v>
-      </c>
-      <c r="B52" s="10" t="s">
-        <v>322</v>
-      </c>
+      <c r="A52" s="9"/>
+      <c r="B52" s="3"/>
       <c r="C52" s="10"/>
       <c r="D52" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>113</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="F52" s="3"/>
       <c r="G52" s="3"/>
-      <c r="H52" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="J52" s="25" t="s">
-        <v>326</v>
-      </c>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="24"/>
       <c r="K52" s="4"/>
       <c r="L52" s="3"/>
       <c r="M52" s="3"/>
-      <c r="N52" s="4" t="s">
+      <c r="N52" s="4"/>
+    </row>
+    <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A53" s="9"/>
-      <c r="B53" s="3"/>
       <c r="C53" s="10"/>
-      <c r="D53" s="3" t="s">
-        <v>328</v>
-      </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
       <c r="I53" s="3"/>
-      <c r="J53" s="25"/>
-      <c r="K53" s="4"/>
+      <c r="J53" s="23"/>
+      <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3"/>
-      <c r="N53" s="4"/>
-    </row>
-    <row r="54" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A54" s="9" t="s">
+      <c r="N53" s="3"/>
+    </row>
+    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="B54" s="10"/>
+      <c r="C54" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="D54" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="C54" s="10"/>
-      <c r="F54" s="3"/>
+      <c r="E54" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="J54" s="24"/>
-      <c r="K54" s="3"/>
-      <c r="L54" s="3"/>
-      <c r="M54" s="3"/>
+      <c r="H54" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="J54" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="K54" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="L54" s="25"/>
+      <c r="M54" s="25"/>
       <c r="N54" s="3"/>
     </row>
-    <row r="55" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="20" t="s">
-        <v>331</v>
-      </c>
-      <c r="B55" s="10"/>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A55" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="B55" s="3"/>
       <c r="C55" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G55" s="3"/>
       <c r="H55" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I55" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="J55" s="21" t="s">
-        <v>336</v>
-      </c>
-      <c r="K55" s="26" t="s">
-        <v>337</v>
-      </c>
-      <c r="L55" s="26"/>
-      <c r="M55" s="26"/>
+        <v>248</v>
+      </c>
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+      <c r="K55" s="25"/>
+      <c r="L55" s="17"/>
+      <c r="M55" s="17"/>
       <c r="N55" s="3"/>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="9" t="s">
-        <v>338</v>
-      </c>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3" t="s">
+    <row r="56" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A56" s="19" t="s">
         <v>339</v>
       </c>
+      <c r="B56" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="C56" s="10"/>
       <c r="D56" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="I56" s="3"/>
-      <c r="J56" s="3"/>
-      <c r="K56" s="26"/>
-      <c r="L56" s="17"/>
-      <c r="M56" s="17"/>
+        <v>91</v>
+      </c>
+      <c r="I56" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="J56" s="20" t="s">
+        <v>344</v>
+      </c>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
       <c r="N56" s="3"/>
     </row>
-    <row r="57" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A57" s="20" t="s">
-        <v>342</v>
+    <row r="57" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="19" t="s">
+        <v>345</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>113</v>
+        <v>349</v>
       </c>
       <c r="G57" s="3"/>
       <c r="H57" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I57" s="34" t="s">
-        <v>346</v>
-      </c>
-      <c r="J57" s="21" t="s">
-        <v>347</v>
+        <v>91</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>351</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
     </row>
-    <row r="58" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="20" t="s">
-        <v>348</v>
-      </c>
-      <c r="B58" s="10" t="s">
-        <v>349</v>
-      </c>
-      <c r="C58" s="10"/>
+    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="19" t="s">
+        <v>352</v>
+      </c>
+      <c r="B58" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="C58" s="27"/>
       <c r="D58" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>351</v>
+        <v>289</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>352</v>
+        <v>161</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="3" t="s">
-        <v>94</v>
+        <v>248</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="3"/>
       <c r="M58" s="3"/>
       <c r="N58" s="3"/>
     </row>
-    <row r="59" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="20" t="s">
-        <v>355</v>
-      </c>
-      <c r="B59" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="C59" s="28"/>
-      <c r="D59" s="3" t="s">
+    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="9" t="s">
         <v>356</v>
       </c>
+      <c r="B59" t="s">
+        <v>357</v>
+      </c>
+      <c r="D59" s="21" t="s">
+        <v>358</v>
+      </c>
       <c r="E59" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="I59" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="J59" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="K59" s="3"/>
-      <c r="L59" s="3"/>
-      <c r="M59" s="3"/>
-      <c r="N59" s="3"/>
-    </row>
-    <row r="60" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="9" t="s">
         <v>359</v>
       </c>
-      <c r="B60" t="s">
+      <c r="H59" t="s">
         <v>360</v>
       </c>
-      <c r="D60" s="22" t="s">
+      <c r="I59" t="s">
         <v>361</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="J59" t="s">
         <v>362</v>
       </c>
-      <c r="H60" t="s">
-        <v>363</v>
-      </c>
-      <c r="I60" t="s">
-        <v>364</v>
-      </c>
-      <c r="J60" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B63" s="28"/>
+      <c r="C63" s="28"/>
+    </row>
+    <row r="64" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
-    </row>
-    <row r="65" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="30"/>
-      <c r="C65" s="31"/>
-    </row>
-    <row r="66" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="29"/>
-      <c r="C66" s="29"/>
+      <c r="C64" s="30"/>
+    </row>
+    <row r="65" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="28"/>
+      <c r="C65" s="28"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="N52" r:id="rId1" xr:uid="{F83F3B55-B4C2-4802-934F-C9E3C14B805B}"/>
-    <hyperlink ref="N24" r:id="rId2" xr:uid="{B73C5555-EF90-4C17-AFEA-F4306780E8B3}"/>
-    <hyperlink ref="N21" r:id="rId3" xr:uid="{FEF2826C-4538-4BD0-84C3-18169970B566}"/>
+    <hyperlink ref="N51" r:id="rId1" xr:uid="{F83F3B55-B4C2-4802-934F-C9E3C14B805B}"/>
+    <hyperlink ref="N23" r:id="rId2" xr:uid="{B73C5555-EF90-4C17-AFEA-F4306780E8B3}"/>
+    <hyperlink ref="N20" r:id="rId3" xr:uid="{FEF2826C-4538-4BD0-84C3-18169970B566}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
@@ -5424,10 +5374,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>64</v>
@@ -5447,25 +5397,25 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -5482,7 +5432,7 @@
     <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -5502,7 +5452,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B1" t="s">
         <v>34</v>
@@ -5510,15 +5460,15 @@
     </row>
     <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -5542,7 +5492,7 @@
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -5550,52 +5500,52 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" s="16" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C3" s="16" t="s">
         <v>56</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="14" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="E4" s="14"/>
     </row>
     <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
+        <v>379</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="19"/>
+      <c r="B6" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>382</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>283</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>383</v>
-      </c>
-      <c r="E5" s="14"/>
-    </row>
-    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>385</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5605,37 +5555,37 @@
     </row>
     <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="14" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C7" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>384</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>387</v>
       </c>
       <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" s="14" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C8" s="14"/>
-      <c r="D8" s="36" t="s">
-        <v>389</v>
+      <c r="D8" s="35" t="s">
+        <v>386</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B9" s="14"/>
       <c r="C9" s="14" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>392</v>
-      </c>
-      <c r="E9" s="24"/>
+        <v>389</v>
+      </c>
+      <c r="E9" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5646,6 +5596,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -5852,17 +5813,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5873,6 +5823,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5891,23 +5858,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Fixed column Beschrijving by moving that title to where the contents are
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Nictiz\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD10C5A-4E46-4677-812B-8C2FB5410E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED832230-90A2-B141-8A59-508F66A307AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-140" yWindow="-26660" windowWidth="43920" windowHeight="26260" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -126,15 +126,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="390">
   <si>
     <t>Veld</t>
   </si>
   <si>
     <t>Beschrijving</t>
-  </si>
-  <si>
-    <t>a.d.h.v. keuze FHIR als basismodel</t>
   </si>
   <si>
     <t>Conceptbeschrijving</t>
@@ -1652,7 +1649,6 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1675,6 +1671,7 @@
       <sz val="9"/>
       <color rgb="FF4D4D4D"/>
       <name val="Tahoma"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1699,7 +1696,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1989,6 +1985,46 @@
       </border>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2054,46 +2090,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment wrapText="1"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2815,44 +2811,44 @@
   <autoFilter ref="A2:C13" xr:uid="{7AAA9086-205B-4EC4-8920-A2DD04D02676}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{BDCFF82A-D4BE-440B-90DF-AA26F6831D5C}" name="Veld"/>
-    <tableColumn id="2" xr3:uid="{77503B9E-152C-4B39-87F4-D4FBBF1B3BDA}" name="Beschrijving" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{B530BE2A-715C-42B8-BFE1-95637D35484B}" name="a.d.h.v. keuze FHIR als basismodel"/>
+    <tableColumn id="2" xr3:uid="{77503B9E-152C-4B39-87F4-D4FBBF1B3BDA}" name="Uitleg" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{B530BE2A-715C-42B8-BFE1-95637D35484B}" name="Beschrijving"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}" name="Tabel3" displayName="Tabel3" ref="A1:E17" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}" name="Tabel3" displayName="Tabel3" ref="A1:E17" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:E17" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2D5F85E5-856C-4A15-8C5D-D8D344B8F13C}" name="Type bron" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{062A7D5A-6D4F-45DD-9A5C-7A2D82A1266A}" name="Naam bron" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{24E64AAE-4BAD-402C-98B7-B46BE371B39E}" name="Toelichting" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{98DE6918-807C-41E0-ACBA-1E2221CF05FC}" name="Informatiebehoefte verwerkt in sheet 'informatiebeheofte'" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{8CFF4D4C-ABDD-49BC-8B49-237193168687}" name="Link naar bron informatie" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{2D5F85E5-856C-4A15-8C5D-D8D344B8F13C}" name="Type bron" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{062A7D5A-6D4F-45DD-9A5C-7A2D82A1266A}" name="Naam bron" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{24E64AAE-4BAD-402C-98B7-B46BE371B39E}" name="Toelichting" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{98DE6918-807C-41E0-ACBA-1E2221CF05FC}" name="Informatiebehoefte verwerkt in sheet 'informatiebeheofte'" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{8CFF4D4C-ABDD-49BC-8B49-237193168687}" name="Link naar bron informatie" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N59" totalsRowShown="0" headerRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N59" totalsRowShown="0" headerRowDxfId="20">
   <autoFilter ref="A2:N59" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="18"/>
     <tableColumn id="12" xr3:uid="{721FE94A-B8C9-44E1-A03C-56E48CDCE2A3}" name="data-element"/>
-    <tableColumn id="3" xr3:uid="{12776FCA-6A89-4E9E-907F-2E30F0D43DA3}" name="Omschrijving" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{9E28C4DB-2A8B-484B-80F1-321440976652}" name="Variabiliteit" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{12776FCA-6A89-4E9E-907F-2E30F0D43DA3}" name="Omschrijving" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{9E28C4DB-2A8B-484B-80F1-321440976652}" name="Variabiliteit" dataDxfId="16"/>
     <tableColumn id="5" xr3:uid="{6FA3E114-7382-4230-B15E-A8DB28B8CE4B}" name="Aanwezigheid"/>
     <tableColumn id="6" xr3:uid="{E8FFDBDF-8B88-4089-89D0-252402D12764}" name="Verleden/heden/toekomst"/>
     <tableColumn id="7" xr3:uid="{BB9C62AB-9839-431A-90A2-B6A6D70DF1FB}" name="Herkomst"/>
     <tableColumn id="8" xr3:uid="{6BE87E7D-EFAE-42FD-9334-11E5EBAC9DC3}" name="Komt het in FHIR R4 voor?"/>
     <tableColumn id="9" xr3:uid="{C6EE00AA-2B37-4BE3-B349-AF61C6E68575}" name="Komt het in openEHR voor?"/>
     <tableColumn id="10" xr3:uid="{943D4BF3-315C-41FB-99E4-8DB8C54604A4}" name="Komt voor in ZIBProbleem-v4.4? (2020)"/>
-    <tableColumn id="14" xr3:uid="{8B1A7EB4-D690-4A36-9698-ACA592C2A715}" name="Komt voor in ZIBProbleem? (2017)" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{51A57E0A-A216-45BB-973D-E0D8C72BEEEC}" name="Komt voor in ZIBProbleem? (2024)" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{8B1A7EB4-D690-4A36-9698-ACA592C2A715}" name="Komt voor in ZIBProbleem? (2017)" dataDxfId="15"/>
+    <tableColumn id="13" xr3:uid="{51A57E0A-A216-45BB-973D-E0D8C72BEEEC}" name="Komt voor in ZIBProbleem? (2024)" dataDxfId="14"/>
     <tableColumn id="11" xr3:uid="{E7EDB106-7E3F-4122-A864-3B3AE59C9D87}" name="Opmerking"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3234,15 +3230,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="218.42578125" customWidth="1"/>
+    <col min="1" max="1" width="218.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18">
         <f>(510*132.5) + (160*132.5)</f>
         <v>88775</v>
@@ -3251,7 +3247,7 @@
         <v>5832</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19">
         <f>(542*132.5)</f>
         <v>71815</v>
@@ -3269,138 +3265,138 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="46.7109375" customWidth="1"/>
-    <col min="3" max="3" width="59.7109375" customWidth="1"/>
+    <col min="2" max="2" width="46.6640625" customWidth="1"/>
+    <col min="3" max="3" width="59.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="219.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="408" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="3" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="3" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="17" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="156" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="3" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="105" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="3" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="5" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B11" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="3" t="s">
+    </row>
+    <row r="12" spans="1:3" ht="256" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="349.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>30</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="3" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="7"/>
     </row>
@@ -3420,214 +3416,214 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8AA88E1-0CFC-4A69-A682-35DA329C9688}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="51.28515625" customWidth="1"/>
-    <col min="3" max="3" width="67.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="51.33203125" customWidth="1"/>
+    <col min="3" max="3" width="67.33203125" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="5" max="5" width="58.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="5" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>54</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="5" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="6"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3654,74 +3650,74 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:O65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" customWidth="1"/>
-    <col min="4" max="4" width="87.42578125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.5" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" customWidth="1"/>
+    <col min="4" max="4" width="87.5" style="3" customWidth="1"/>
     <col min="5" max="5" width="78" style="3" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" customWidth="1"/>
-    <col min="8" max="8" width="32.42578125" customWidth="1"/>
-    <col min="9" max="9" width="28.140625" customWidth="1"/>
-    <col min="10" max="10" width="51.28515625" customWidth="1"/>
-    <col min="11" max="11" width="38.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="38.5703125" customWidth="1"/>
-    <col min="14" max="14" width="33.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.5" customWidth="1"/>
+    <col min="8" max="8" width="32.5" customWidth="1"/>
+    <col min="9" max="9" width="28.1640625" customWidth="1"/>
+    <col min="10" max="10" width="51.33203125" customWidth="1"/>
+    <col min="11" max="11" width="38.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="38.5" customWidth="1"/>
+    <col min="14" max="14" width="33.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
         <v>63</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>64</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="J2" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="K2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>81</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>82</v>
       </c>
       <c r="C3" s="18"/>
       <c r="D3" s="19"/>
@@ -3730,42 +3726,42 @@
       <c r="G3" s="19"/>
       <c r="H3" s="19"/>
       <c r="I3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="K3" s="19" t="s">
-        <v>85</v>
-      </c>
       <c r="L3" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M3" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N3" s="19"/>
       <c r="O3" s="9"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -3774,26 +3770,26 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
     </row>
-    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="F5" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -3802,26 +3798,26 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>99</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -3830,26 +3826,26 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="80" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="E7" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -3858,16 +3854,16 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="26" t="s">
         <v>104</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>105</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -3879,244 +3875,244 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I9" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="L9" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="64" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>120</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>121</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I11" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="J11" s="23" t="s">
+      <c r="K11" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="L11" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="96" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>132</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I12" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="J12" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="3" t="s">
-        <v>135</v>
-      </c>
       <c r="K12" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>140</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="J13" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K13" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="L13" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>147</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="E15" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>152</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="I15" s="3" t="s">
-        <v>154</v>
-      </c>
       <c r="J15" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>155</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>156</v>
       </c>
       <c r="C16" s="3"/>
       <c r="F16" s="3"/>
@@ -4129,60 +4125,60 @@
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I17" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="J17" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="J17" s="32" t="s">
-        <v>163</v>
-      </c>
       <c r="K17" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>167</v>
-      </c>
       <c r="F18" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
@@ -4191,16 +4187,16 @@
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B19" s="22" t="s">
         <v>169</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>170</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -4212,81 +4208,81 @@
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="E20" s="37" t="s">
-        <v>175</v>
-      </c>
       <c r="F20" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I20" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="J20" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="J20" s="20" t="s">
+      <c r="K20" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>178</v>
       </c>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
       <c r="N20" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="19" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="C21" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>182</v>
-      </c>
       <c r="F21" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>184</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>185</v>
       </c>
       <c r="C22" s="10"/>
       <c r="F22" s="3"/>
@@ -4299,66 +4295,66 @@
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>189</v>
-      </c>
       <c r="F23" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I23" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="J23" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="J23" s="23" t="s">
+      <c r="K23" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="L23" s="36" t="s">
         <v>192</v>
       </c>
-      <c r="L23" s="36" t="s">
+      <c r="M23" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="M23" s="3" t="s">
+      <c r="N23" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="N23" s="5" t="s">
+    </row>
+    <row r="24" spans="1:14" ht="80" x14ac:dyDescent="0.2">
+      <c r="A24" s="9" t="s">
         <v>195</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="75" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="F24" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I24" s="38"/>
       <c r="J24" s="23"/>
@@ -4367,26 +4363,26 @@
       <c r="M24" s="3"/>
       <c r="N24" s="5"/>
     </row>
-    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="D25" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="D25" s="37" t="s">
+      <c r="E25" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="E25" s="37" t="s">
-        <v>203</v>
-      </c>
       <c r="F25" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I25" s="3"/>
       <c r="J25" s="23"/>
@@ -4395,108 +4391,108 @@
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
-    <row r="26" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A26" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>205</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>206</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>208</v>
-      </c>
       <c r="F26" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I26" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="J26" s="3" t="s">
-        <v>210</v>
-      </c>
       <c r="K26" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="B27" s="22" t="s">
         <v>211</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>212</v>
       </c>
       <c r="C27" s="22"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="J27" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="J27" s="3" t="s">
+      <c r="K27" s="3" t="s">
         <v>214</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>215</v>
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="F28" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I28" s="3"/>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>223</v>
-      </c>
       <c r="F29" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
@@ -4505,26 +4501,26 @@
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="F30" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
@@ -4533,26 +4529,26 @@
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>232</v>
-      </c>
       <c r="F31" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
@@ -4561,78 +4557,78 @@
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
     </row>
-    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" s="10" t="s">
         <v>234</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>235</v>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H32" s="3"/>
       <c r="I32" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J32" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="K32" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>240</v>
       </c>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="19" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>243</v>
-      </c>
       <c r="E33" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>247</v>
-      </c>
       <c r="F34" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="31"/>
@@ -4641,26 +4637,26 @@
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>252</v>
-      </c>
       <c r="F35" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
@@ -4669,81 +4665,81 @@
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B36" s="10" t="s">
         <v>254</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>255</v>
       </c>
       <c r="C36" s="10"/>
       <c r="D36" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="H36" s="3"/>
       <c r="I36" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="J36" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>259</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="19" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>262</v>
-      </c>
       <c r="E37" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="E38" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="E38" s="3" t="s">
-        <v>267</v>
-      </c>
       <c r="F38" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
@@ -4752,26 +4748,26 @@
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="34" t="s">
+        <v>268</v>
+      </c>
+      <c r="D39" s="17" t="s">
         <v>269</v>
       </c>
-      <c r="D39" s="17" t="s">
-        <v>270</v>
-      </c>
       <c r="E39" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
@@ -4780,59 +4776,59 @@
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="19" t="s">
+        <v>271</v>
+      </c>
+      <c r="B40" s="10" t="s">
         <v>272</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>273</v>
       </c>
       <c r="C40" s="10"/>
       <c r="D40" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I40" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="J40" s="20" t="s">
         <v>275</v>
-      </c>
-      <c r="J40" s="20" t="s">
-        <v>276</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="10"/>
       <c r="D41" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>279</v>
-      </c>
       <c r="F41" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
@@ -4840,72 +4836,72 @@
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B42" s="3"/>
       <c r="C42" s="10"/>
       <c r="D42" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E42" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="E42" s="3" t="s">
-        <v>283</v>
-      </c>
       <c r="F42" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
     </row>
-    <row r="43" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="B43" s="10" t="s">
         <v>286</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>287</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>289</v>
-      </c>
       <c r="F43" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I43" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="J43" s="33" t="s">
         <v>290</v>
-      </c>
-      <c r="J43" s="33" t="s">
-        <v>291</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
     </row>
-    <row r="44" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="3"/>
       <c r="C44" s="10"/>
       <c r="D44" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -4917,48 +4913,48 @@
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="B45" s="10" t="s">
         <v>293</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>294</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E45" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="F45" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G45" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="F45" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="G45" s="3" t="s">
+      <c r="H45" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I45" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="H45" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I45" s="3" t="s">
+      <c r="J45" s="3" t="s">
         <v>298</v>
-      </c>
-      <c r="J45" s="3" t="s">
-        <v>299</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B46" s="3"/>
       <c r="C46" s="10"/>
       <c r="D46" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -4970,26 +4966,26 @@
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
-    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B47" s="3"/>
       <c r="C47" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="D47" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="E47" s="3" t="s">
         <v>304</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>305</v>
       </c>
       <c r="F47" s="3">
         <v>1</v>
       </c>
       <c r="G47" s="3"/>
       <c r="H47" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
@@ -4998,55 +4994,55 @@
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="B48" s="10" t="s">
         <v>306</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>307</v>
       </c>
       <c r="C48" s="10"/>
       <c r="D48" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="E48" s="3" t="s">
-        <v>309</v>
-      </c>
       <c r="F48" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G48" s="3"/>
       <c r="H48" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I48" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="J48" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="J48" s="3" t="s">
-        <v>311</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B49" s="3"/>
       <c r="C49" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="D49" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>314</v>
-      </c>
       <c r="F49" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
@@ -5055,23 +5051,23 @@
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
     </row>
-    <row r="50" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="19" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B50" s="3"/>
       <c r="C50" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D50" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="D50" s="3" t="s">
-        <v>317</v>
-      </c>
       <c r="F50" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I50" s="3"/>
       <c r="J50" s="3"/>
@@ -5080,46 +5076,46 @@
       <c r="M50" s="3"/>
       <c r="N50" s="3"/>
     </row>
-    <row r="51" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="19" t="s">
+        <v>317</v>
+      </c>
+      <c r="B51" s="10" t="s">
         <v>318</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>319</v>
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="E51" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="E51" s="3" t="s">
-        <v>321</v>
-      </c>
       <c r="F51" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I51" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="J51" s="24" t="s">
         <v>322</v>
-      </c>
-      <c r="J51" s="24" t="s">
-        <v>323</v>
       </c>
       <c r="K51" s="4"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
       <c r="N51" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A52" s="9"/>
       <c r="B52" s="3"/>
       <c r="C52" s="10"/>
       <c r="D52" s="3" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -5131,12 +5127,12 @@
       <c r="M52" s="3"/>
       <c r="N52" s="4"/>
     </row>
-    <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>326</v>
-      </c>
-      <c r="B53" s="10" t="s">
-        <v>327</v>
       </c>
       <c r="C53" s="10"/>
       <c r="F53" s="3"/>
@@ -5149,60 +5145,60 @@
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
     </row>
-    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B54" s="10"/>
       <c r="C54" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="D54" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="E54" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="E54" s="3" t="s">
-        <v>331</v>
-      </c>
       <c r="F54" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G54" s="3"/>
       <c r="H54" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I54" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="J54" s="20" t="s">
         <v>332</v>
       </c>
-      <c r="J54" s="20" t="s">
+      <c r="K54" s="25" t="s">
         <v>333</v>
-      </c>
-      <c r="K54" s="25" t="s">
-        <v>334</v>
       </c>
       <c r="L54" s="25"/>
       <c r="M54" s="25"/>
       <c r="N54" s="3"/>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="D55" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="E55" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="E55" s="3" t="s">
-        <v>338</v>
-      </c>
       <c r="F55" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G55" s="3"/>
       <c r="H55" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I55" s="3"/>
       <c r="J55" s="3"/>
@@ -5211,134 +5207,134 @@
       <c r="M55" s="17"/>
       <c r="N55" s="3"/>
     </row>
-    <row r="56" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A56" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="B56" s="10" t="s">
         <v>339</v>
-      </c>
-      <c r="B56" s="10" t="s">
-        <v>340</v>
       </c>
       <c r="C56" s="10"/>
       <c r="D56" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="E56" s="3" t="s">
-        <v>342</v>
-      </c>
       <c r="F56" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I56" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="J56" s="20" t="s">
         <v>343</v>
-      </c>
-      <c r="J56" s="20" t="s">
-        <v>344</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="3"/>
       <c r="N56" s="3"/>
     </row>
-    <row r="57" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="B57" s="10" t="s">
         <v>345</v>
-      </c>
-      <c r="B57" s="10" t="s">
-        <v>346</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="E57" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="E57" s="3" t="s">
+      <c r="F57" s="3" t="s">
         <v>348</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>349</v>
       </c>
       <c r="G57" s="3"/>
       <c r="H57" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I57" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J57" s="3" t="s">
         <v>350</v>
-      </c>
-      <c r="J57" s="3" t="s">
-        <v>351</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
     </row>
-    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="19" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B58" s="27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C58" s="27"/>
       <c r="D58" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I58" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="J58" s="3" t="s">
         <v>354</v>
-      </c>
-      <c r="J58" s="3" t="s">
-        <v>355</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="3"/>
       <c r="M58" s="3"/>
       <c r="N58" s="3"/>
     </row>
-    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="B59" t="s">
         <v>356</v>
       </c>
-      <c r="B59" t="s">
+      <c r="D59" s="21" t="s">
         <v>357</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="E59" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="H59" t="s">
         <v>359</v>
       </c>
-      <c r="H59" t="s">
+      <c r="I59" t="s">
         <v>360</v>
       </c>
-      <c r="I59" t="s">
+      <c r="J59" t="s">
         <v>361</v>
       </c>
-      <c r="J59" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B63" s="28"/>
       <c r="C63" s="28"/>
     </row>
-    <row r="64" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B64" s="29"/>
       <c r="C64" s="30"/>
     </row>
-    <row r="65" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B65" s="28"/>
       <c r="C65" s="28"/>
     </row>
@@ -5362,60 +5358,60 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="41.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19.1640625" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="4" max="4" width="15.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
+    <col min="7" max="7" width="41.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>367</v>
-      </c>
       <c r="D2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -5427,12 +5423,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -5444,31 +5440,31 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0062C35-A590-498D-8635-16DE3DC0B82A}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="36.5703125" customWidth="1"/>
+    <col min="1" max="1" width="36.5" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>370</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -5482,70 +5478,70 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E8E4E8-143C-4C64-99FB-1306F2338EFB}">
   <dimension ref="A2:J9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="27.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="60.140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="47.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="27.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="60.1640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="47.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="15" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B3" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>373</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="16" t="s">
+      <c r="E3" s="13" t="s">
         <v>374</v>
       </c>
-      <c r="E3" s="13" t="s">
+    </row>
+    <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="14" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>376</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>379</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>380</v>
-      </c>
       <c r="E5" s="14"/>
     </row>
-    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>381</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>382</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5553,37 +5549,37 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B7" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>380</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="14"/>
+    </row>
+    <row r="8" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="B8" s="14" t="s">
         <v>384</v>
-      </c>
-      <c r="E7" s="14"/>
-    </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B8" s="14" t="s">
-        <v>385</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="35" t="s">
+        <v>385</v>
+      </c>
+      <c r="E8" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="E8" s="14" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="B9" s="14"/>
       <c r="C9" s="14" t="s">
+        <v>387</v>
+      </c>
+      <c r="D9" s="14" t="s">
         <v>388</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>389</v>
       </c>
       <c r="E9" s="23"/>
     </row>
@@ -5607,6 +5603,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -5813,15 +5818,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
@@ -5840,6 +5836,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5856,12 +5860,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>